<commit_message>
De-duplicate Tata issue-policy failures (by proposal) and CarrierPolicyNo cases (by policy)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H8J8gdeYPbiAaQWCg6AHZG
</commit_message>
<xml_diff>
--- a/september-2026/failure-logs-12-21Oct2026/Tata_CarrierPolicyNo_Cases_with_Logs_Jul-Oct2026.xlsx
+++ b/september-2026/failure-logs-12-21Oct2026/Tata_CarrierPolicyNo_Cases_with_Logs_Jul-Oct2026.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:N24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -462,6 +462,8 @@
     <col width="60" customWidth="1" min="10" max="10"/>
     <col width="60" customWidth="1" min="11" max="11"/>
     <col width="60" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -525,6 +527,16 @@
           <t>InsureMO response</t>
         </is>
       </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Calls with this CarrierPolicyNo</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Last call</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -585,16 +597,24 @@
           <t>{"ClientRequestId": "4f71a456-2465-44b6-b7ad-5d4c6a90bed1", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6170596719-00", "CarrierProposalNo": "PR/26/6170466062", "CarrierQuoteRequestId": "QT/26/6175204126", "InspectionId": "N500001649699", "PaymentId": "6fab06aa9a6946a4d443f24221218241:38f7c75cf1da2c2bff32c1b13d180ecb", "requestId": "P500185782652"}, "ResultCode": 1, "TransactionType": 2003}</t>
         </is>
       </c>
+      <c r="M2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06T01:38:44</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06T01:38:44</t>
+          <t>2026-07-09T14:05:59</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
@@ -602,17 +622,17 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>6170596719-00</t>
+          <t>6170607023-00</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>a2a12c8a59439513e758683c1629f631</t>
+          <t>1fdde7c2a6533eae097ce404d3e69b7e</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>9eba2394-6377-4403-b1e4-9a411da663e8</t>
+          <t>d8d4bd3c-df58-40dc-924d-bdb3e1071843</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -627,34 +647,42 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6170466062", "EffectiveDate": "2026-07-06", "PolicyPaymentInfoList": [{"Amount": "1241", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-07-06T01:38:43", "TransactionId": "04a7a8f0160e9334bd3cff0f98cd4eb6:a73c2c5282df41fbaa6297fd6d9c3dca", "TransactionNo": "T9wojMtOcTNq7k"}]}</t>
+          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6170480774", "EffectiveDate": "2026-07-09", "PolicyPaymentInfoList": [{"Amount": "895", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-07-09T14:05:59", "TransactionId": "aef2543408c477eb052f799a5892d979:9bc85fbcf440712d10399f53b85f83ee", "TransactionNo": "TBL8tmwrdajT2x"}]}</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6170466062", "EffectiveDate": "2026-07-06", "PolicyPaymentInfoList": [{"Amount": "1241", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-07-06T01:38:43", "TransactionId": "04a7a8f0160e9334bd3cff0f98cd4eb6:a73c2c5282df41fbaa6297fd6d9c3dca", "TransactionNo": "T9wojMtOcTNq7k"}]}</t>
+          <t>{"ihub.body": {"consumerAppTransId": "TBL8tmwrdajT2x", "gateway_txn_id": "TBL8tmwrdajT2x", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "895", "payment_id": "aef2543408c477eb052f799a5892d979:9bc85fbcf440712d10399f53b85f83ee", "policy_start_date": "2026-07-09", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-07-09 14:05:59"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>{"CarrierCode": "25", "CarrierPolicyNo": "6170596719-00", "CarrierProposalNo": "PR/26/6170466062", "CarrierQuoteRequestId": "QT/26/6175204126", "InspectionId": "N500001649699", "PaymentId": "8175d32878dbe42b93d3c7e34686c0e6:b8f1b76e208b8e6b54e9a3d7a7e9a90e", "requestId": "P500185782652"}</t>
+          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "a3b92a9d90c4c7d4eb38ef0195c53d02:89b46be0d4bcc5ab81d1a28555ff5eec", "encrypted_policy_no": "a8ff89b6c90d2e2eec6ad07bed192c22:d619f6c1f0f39816f014999ff24d25dd", "master_policy": "", "net_premium": 895, "nstp_id": "N500001672601", "nstp_stage": "completed", "payment_id": "038d65c96c3bdf625ff2c65fb871be53:0c4a2a75f5b1cd8c82ec3c7ef483a18f", "payment_stage": "completed", "policy_id": "P500187182007", "policy_no": "6170607023-00", "product_id": "M300000000002", "proposal_no": "PR/26/6170480774", "proposal_stage": "completed", "quote_no": "QT/26/6175305915", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>{"ClientRequestId": "9eba2394-6377-4403-b1e4-9a411da663e8", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6170596719-00", "CarrierProposalNo": "PR/26/6170466062", "CarrierQuoteRequestId": "QT/26/6175204126", "InspectionId": "N500001649699", "PaymentId": "8175d32878dbe42b93d3c7e34686c0e6:b8f1b76e208b8e6b54e9a3d7a7e9a90e", "requestId": "P500185782652"}, "ResultCode": 1, "TransactionType": 2003}</t>
+          <t>{"ClientRequestId": "d8d4bd3c-df58-40dc-924d-bdb3e1071843", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6170607023-00", "CarrierProposalNo": "PR/26/6170480774", "CarrierQuoteRequestId": "QT/26/6175305915", "InspectionId": "N500001672601", "PaymentId": "038d65c96c3bdf625ff2c65fb871be53:0c4a2a75f5b1cd8c82ec3c7ef483a18f", "requestId": "P500187182007"}, "ResultCode": 1, "TransactionType": 2003}</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09T14:05:59</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09T14:05:59</t>
+          <t>2026-07-11T16:45:02</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
@@ -662,17 +690,17 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>6170607023-00</t>
+          <t>6270421436-00</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>1fdde7c2a6533eae097ce404d3e69b7e</t>
+          <t>123fa5dccd27bf16fefacd8c1ae6fd39</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>d8d4bd3c-df58-40dc-924d-bdb3e1071843</t>
+          <t>59cd5ac1-2795-402d-84b0-282fe78b1b0d</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -687,34 +715,42 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6170480774", "EffectiveDate": "2026-07-09", "PolicyPaymentInfoList": [{"Amount": "895", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-07-09T14:05:59", "TransactionId": "aef2543408c477eb052f799a5892d979:9bc85fbcf440712d10399f53b85f83ee", "TransactionNo": "TBL8tmwrdajT2x"}]}</t>
+          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6270400604", "EffectiveDate": "2026-07-12", "PolicyPaymentInfoList": [{"Amount": "4473", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-07-11T16:45:01", "TransactionId": "fbe8544b71b1dd47931ce4492e459cdf:774cfd5e83f7e7645df4c064965bebdb", "TransactionNo": "TCAvTv8mKBtXey"}]}</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>{"ihub.body": {"consumerAppTransId": "TBL8tmwrdajT2x", "gateway_txn_id": "TBL8tmwrdajT2x", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "895", "payment_id": "aef2543408c477eb052f799a5892d979:9bc85fbcf440712d10399f53b85f83ee", "policy_start_date": "2026-07-09", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-07-09 14:05:59"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
+          <t>{"ihub.body": {"consumerAppTransId": "TCAvTv8mKBtXey", "gateway_txn_id": "TCAvTv8mKBtXey", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "4473", "payment_id": "fbe8544b71b1dd47931ce4492e459cdf:774cfd5e83f7e7645df4c064965bebdb", "policy_start_date": "2026-07-12", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-07-11 16:45:01"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "a3b92a9d90c4c7d4eb38ef0195c53d02:89b46be0d4bcc5ab81d1a28555ff5eec", "encrypted_policy_no": "a8ff89b6c90d2e2eec6ad07bed192c22:d619f6c1f0f39816f014999ff24d25dd", "master_policy": "", "net_premium": 895, "nstp_id": "N500001672601", "nstp_stage": "completed", "payment_id": "038d65c96c3bdf625ff2c65fb871be53:0c4a2a75f5b1cd8c82ec3c7ef483a18f", "payment_stage": "completed", "policy_id": "P500187182007", "policy_no": "6170607023-00", "product_id": "M300000000002", "proposal_no": "PR/26/6170480774", "proposal_stage": "completed", "quote_no": "QT/26/6175305915", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
+          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "7df1ab9140755546ab1ef3d8ece17e4d:dd170f1fa51bcf0049ee4147eb5d0cc9", "encrypted_policy_no": "4842961e863766bc4c8deb21422b7994:1ab01f6b8425c1c34652d0b4a09718ae", "master_policy": "", "net_premium": 4473, "nstp_id": "N500001687064", "nstp_stage": "completed", "payment_id": "b956354ff0f0143ce64954523999e38d:e8674c53d8299362e04e977d5bfc0a53", "payment_stage": "completed", "policy_id": "P500188022067", "policy_no": "6270421436-00", "product_id": "M300000000001", "proposal_no": "PR/26/6270400604", "proposal_stage": "completed", "quote_no": "QT/26/6284535489", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>{"ClientRequestId": "d8d4bd3c-df58-40dc-924d-bdb3e1071843", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6170607023-00", "CarrierProposalNo": "PR/26/6170480774", "CarrierQuoteRequestId": "QT/26/6175305915", "InspectionId": "N500001672601", "PaymentId": "038d65c96c3bdf625ff2c65fb871be53:0c4a2a75f5b1cd8c82ec3c7ef483a18f", "requestId": "P500187182007"}, "ResultCode": 1, "TransactionType": 2003}</t>
+          <t>{"ClientRequestId": "59cd5ac1-2795-402d-84b0-282fe78b1b0d", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6270421436-00", "CarrierProposalNo": "PR/26/6270400604", "CarrierQuoteRequestId": "QT/26/6284535489", "InspectionId": "N500001687064", "PaymentId": "b956354ff0f0143ce64954523999e38d:e8674c53d8299362e04e977d5bfc0a53", "requestId": "P500188022067"}, "ResultCode": 1, "TransactionType": 2003}</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11T16:45:02</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11T16:45:02</t>
+          <t>2026-07-22T15:43:26</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
@@ -722,17 +758,17 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>6270421436-00</t>
+          <t>6270435712-00</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>123fa5dccd27bf16fefacd8c1ae6fd39</t>
+          <t>dfa6f29fe5349a71f0dc3f505ffd43e3</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>59cd5ac1-2795-402d-84b0-282fe78b1b0d</t>
+          <t>c57f11ee-8cfd-428c-a756-618750206256</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -747,34 +783,42 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6270400604", "EffectiveDate": "2026-07-12", "PolicyPaymentInfoList": [{"Amount": "4473", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-07-11T16:45:01", "TransactionId": "fbe8544b71b1dd47931ce4492e459cdf:774cfd5e83f7e7645df4c064965bebdb", "TransactionNo": "TCAvTv8mKBtXey"}]}</t>
+          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6270422086", "EffectiveDate": "2026-08-02", "PolicyPaymentInfoList": [{"Amount": "5308", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-07-22T15:43:26", "TransactionId": "7c2b7bd2970526b7b17b607a5a8ab65a:380dfdaef02feecf8844dd4152cb507d", "TransactionNo": "TGVkRdc8PEvQ8z"}]}</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>{"ihub.body": {"consumerAppTransId": "TCAvTv8mKBtXey", "gateway_txn_id": "TCAvTv8mKBtXey", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "4473", "payment_id": "fbe8544b71b1dd47931ce4492e459cdf:774cfd5e83f7e7645df4c064965bebdb", "policy_start_date": "2026-07-12", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-07-11 16:45:01"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
+          <t>{"ihub.body": {"consumerAppTransId": "TGVkRdc8PEvQ8z", "gateway_txn_id": "TGVkRdc8PEvQ8z", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "5308", "payment_id": "7c2b7bd2970526b7b17b607a5a8ab65a:380dfdaef02feecf8844dd4152cb507d", "policy_start_date": "2026-08-02", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-07-22 15:43:26"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "7df1ab9140755546ab1ef3d8ece17e4d:dd170f1fa51bcf0049ee4147eb5d0cc9", "encrypted_policy_no": "4842961e863766bc4c8deb21422b7994:1ab01f6b8425c1c34652d0b4a09718ae", "master_policy": "", "net_premium": 4473, "nstp_id": "N500001687064", "nstp_stage": "completed", "payment_id": "b956354ff0f0143ce64954523999e38d:e8674c53d8299362e04e977d5bfc0a53", "payment_stage": "completed", "policy_id": "P500188022067", "policy_no": "6270421436-00", "product_id": "M300000000001", "proposal_no": "PR/26/6270400604", "proposal_stage": "completed", "quote_no": "QT/26/6284535489", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
+          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "00cce94b51bd5d1f81a5b35f50bc8d24:4d68467b6f4ced563ae954489557f98a", "encrypted_policy_no": "4f3a70c0e75495be15b866d1beb5aa85:b92bc224c2e69560e33b8c49a3c89b7c", "master_policy": "", "net_premium": 5308, "nstp_id": "N500001756333", "nstp_stage": "completed", "payment_id": "c2fdbd29945eb1b3b3e753799d54a4a3:6f65c38addd288ae6a85274a61a4fad4", "payment_stage": "completed", "policy_id": "P500192088552", "policy_no": "6270435712-00", "product_id": "M300000000001", "proposal_no": "PR/26/6270422086", "proposal_stage": "completed", "quote_no": "QT/26/6285221138", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>{"ClientRequestId": "59cd5ac1-2795-402d-84b0-282fe78b1b0d", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6270421436-00", "CarrierProposalNo": "PR/26/6270400604", "CarrierQuoteRequestId": "QT/26/6284535489", "InspectionId": "N500001687064", "PaymentId": "b956354ff0f0143ce64954523999e38d:e8674c53d8299362e04e977d5bfc0a53", "requestId": "P500188022067"}, "ResultCode": 1, "TransactionType": 2003}</t>
+          <t>{"ClientRequestId": "c57f11ee-8cfd-428c-a756-618750206256", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6270435712-00", "CarrierProposalNo": "PR/26/6270422086", "CarrierQuoteRequestId": "QT/26/6285221138", "InspectionId": "N500001756333", "PaymentId": "c2fdbd29945eb1b3b3e753799d54a4a3:6f65c38addd288ae6a85274a61a4fad4", "requestId": "P500192088552"}, "ResultCode": 1, "TransactionType": 2003}</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22T15:43:26</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-22T15:43:26</t>
+          <t>2026-07-23T17:13:09</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
@@ -782,17 +826,17 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>6270435712-00</t>
+          <t>6170645852-00</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>dfa6f29fe5349a71f0dc3f505ffd43e3</t>
+          <t>87c18ed46697fb50e8a0e23b9f940867</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>c57f11ee-8cfd-428c-a756-618750206256</t>
+          <t>50da1383-af53-4887-b80d-dc835fa8f292</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -807,34 +851,42 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6270422086", "EffectiveDate": "2026-08-02", "PolicyPaymentInfoList": [{"Amount": "5308", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-07-22T15:43:26", "TransactionId": "7c2b7bd2970526b7b17b607a5a8ab65a:380dfdaef02feecf8844dd4152cb507d", "TransactionNo": "TGVkRdc8PEvQ8z"}]}</t>
+          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6170538668", "EffectiveDate": "2026-07-24", "PolicyPaymentInfoList": [{"Amount": "843", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-07-23T17:13:08", "TransactionId": "8cdc2ca9ba9de20f7a76e3a80cfa4d67:d2d6f172ebdac02bbf4eb1516cc2ea94", "TransactionNo": "TGvodE2jEoEeU8"}]}</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>{"ihub.body": {"consumerAppTransId": "TGVkRdc8PEvQ8z", "gateway_txn_id": "TGVkRdc8PEvQ8z", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "5308", "payment_id": "7c2b7bd2970526b7b17b607a5a8ab65a:380dfdaef02feecf8844dd4152cb507d", "policy_start_date": "2026-08-02", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-07-22 15:43:26"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
+          <t>{"ihub.body": {"consumerAppTransId": "TGvodE2jEoEeU8", "gateway_txn_id": "TGvodE2jEoEeU8", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "843", "payment_id": "8cdc2ca9ba9de20f7a76e3a80cfa4d67:d2d6f172ebdac02bbf4eb1516cc2ea94", "policy_start_date": "2026-07-24", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-07-23 17:13:08"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "00cce94b51bd5d1f81a5b35f50bc8d24:4d68467b6f4ced563ae954489557f98a", "encrypted_policy_no": "4f3a70c0e75495be15b866d1beb5aa85:b92bc224c2e69560e33b8c49a3c89b7c", "master_policy": "", "net_premium": 5308, "nstp_id": "N500001756333", "nstp_stage": "completed", "payment_id": "c2fdbd29945eb1b3b3e753799d54a4a3:6f65c38addd288ae6a85274a61a4fad4", "payment_stage": "completed", "policy_id": "P500192088552", "policy_no": "6270435712-00", "product_id": "M300000000001", "proposal_no": "PR/26/6270422086", "proposal_stage": "completed", "quote_no": "QT/26/6285221138", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
+          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "33a49dcc664785de5c2b6efb347f017e:e6cade5bf04f8b708b47a7857340bec8", "encrypted_policy_no": "22c9b31dc65e71ad5664ec83dce03b10:83b4aea4a57953918b94bd1756962fae", "master_policy": "", "net_premium": 843, "nstp_id": "N500001763548", "nstp_stage": "completed", "payment_id": "d15b97742b1d9a2d43b715cc0f13fc07:8a74467e679fecc9eff3f1437617382e", "payment_stage": "completed", "policy_id": "P500192556250", "policy_no": "6170645852-00", "product_id": "M300000000002", "proposal_no": "PR/26/6170538668", "proposal_stage": "completed", "quote_no": "QT/26/6175687549", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>{"ClientRequestId": "c57f11ee-8cfd-428c-a756-618750206256", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6270435712-00", "CarrierProposalNo": "PR/26/6270422086", "CarrierQuoteRequestId": "QT/26/6285221138", "InspectionId": "N500001756333", "PaymentId": "c2fdbd29945eb1b3b3e753799d54a4a3:6f65c38addd288ae6a85274a61a4fad4", "requestId": "P500192088552"}, "ResultCode": 1, "TransactionType": 2003}</t>
+          <t>{"ClientRequestId": "50da1383-af53-4887-b80d-dc835fa8f292", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6170645852-00", "CarrierProposalNo": "PR/26/6170538668", "CarrierQuoteRequestId": "QT/26/6175687549", "InspectionId": "N500001763548", "PaymentId": "d15b97742b1d9a2d43b715cc0f13fc07:8a74467e679fecc9eff3f1437617382e", "requestId": "P500192556250"}, "ResultCode": 1, "TransactionType": 2003}</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-23T17:13:10</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-23T17:13:09</t>
+          <t>2026-08-04T23:57:09</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
@@ -842,17 +894,17 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>6170645852-00</t>
+          <t>6170677969-00</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>87c18ed46697fb50e8a0e23b9f940867</t>
+          <t>0ce36c7d775e8f96d4ceed2a617f9518</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>50da1383-af53-4887-b80d-dc835fa8f292</t>
+          <t>6db2e587-29f8-4264-890d-97d3fd8d2a44</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -867,34 +919,42 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6170538668", "EffectiveDate": "2026-07-24", "PolicyPaymentInfoList": [{"Amount": "843", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-07-23T17:13:08", "TransactionId": "8cdc2ca9ba9de20f7a76e3a80cfa4d67:d2d6f172ebdac02bbf4eb1516cc2ea94", "TransactionNo": "TGvodE2jEoEeU8"}]}</t>
+          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6170589741", "EffectiveDate": "2026-08-05", "PolicyPaymentInfoList": [{"Amount": "1374", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-08-04T23:57:08", "TransactionId": "3e93982a459ab3689910ea9fd1e19117:af925455d51084d8172a835b3364b531", "TransactionNo": "TLn6gZDOXDNPga"}]}</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>{"ihub.body": {"consumerAppTransId": "TGvodE2jEoEeU8", "gateway_txn_id": "TGvodE2jEoEeU8", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "843", "payment_id": "8cdc2ca9ba9de20f7a76e3a80cfa4d67:d2d6f172ebdac02bbf4eb1516cc2ea94", "policy_start_date": "2026-07-24", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-07-23 17:13:08"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
+          <t>{"ihub.body": {"consumerAppTransId": "TLn6gZDOXDNPga", "gateway_txn_id": "TLn6gZDOXDNPga", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "1374", "payment_id": "3e93982a459ab3689910ea9fd1e19117:af925455d51084d8172a835b3364b531", "policy_start_date": "2026-08-05", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-08-04 23:57:08"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "33a49dcc664785de5c2b6efb347f017e:e6cade5bf04f8b708b47a7857340bec8", "encrypted_policy_no": "22c9b31dc65e71ad5664ec83dce03b10:83b4aea4a57953918b94bd1756962fae", "master_policy": "", "net_premium": 843, "nstp_id": "N500001763548", "nstp_stage": "completed", "payment_id": "d15b97742b1d9a2d43b715cc0f13fc07:8a74467e679fecc9eff3f1437617382e", "payment_stage": "completed", "policy_id": "P500192556250", "policy_no": "6170645852-00", "product_id": "M300000000002", "proposal_no": "PR/26/6170538668", "proposal_stage": "completed", "quote_no": "QT/26/6175687549", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
+          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "a138ecac97d25d04f9b697cb90bbd8cd:558503a1be3105fe0865b0a5dd933efa", "encrypted_policy_no": "d64c856525a014021b8819c8921aca5f:5c1e9c90f490b008202d036ed9ca9350", "master_policy": "", "net_premium": 1374, "nstp_id": "N500001843894", "nstp_stage": "completed", "payment_id": "8422f8f1c61551c6512f9b2f5116f92d:221334417c936d8c0d93c8dfce0b8732", "payment_stage": "completed", "policy_id": "P500197370675", "policy_no": "6170677969-00", "product_id": "M300000000002", "proposal_no": "PR/26/6170589741", "proposal_stage": "completed", "quote_no": "QT/26/6176022411", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>{"ClientRequestId": "50da1383-af53-4887-b80d-dc835fa8f292", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6170645852-00", "CarrierProposalNo": "PR/26/6170538668", "CarrierQuoteRequestId": "QT/26/6175687549", "InspectionId": "N500001763548", "PaymentId": "d15b97742b1d9a2d43b715cc0f13fc07:8a74467e679fecc9eff3f1437617382e", "requestId": "P500192556250"}, "ResultCode": 1, "TransactionType": 2003}</t>
+          <t>{"ClientRequestId": "6db2e587-29f8-4264-890d-97d3fd8d2a44", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6170677969-00", "CarrierProposalNo": "PR/26/6170589741", "CarrierQuoteRequestId": "QT/26/6176022411", "InspectionId": "N500001843894", "PaymentId": "8422f8f1c61551c6512f9b2f5116f92d:221334417c936d8c0d93c8dfce0b8732", "requestId": "P500197370675"}, "ResultCode": 1, "TransactionType": 2003}</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-04T23:57:15</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-23T17:13:10</t>
+          <t>2026-08-05T20:51:49</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
@@ -902,17 +962,17 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>6170645852-00</t>
+          <t>6170681150-00</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>64e154dde1d1072e276226309f1e1bf6</t>
+          <t>ada238190acdde9e08489db376da2ffc</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>62da7d91-33f9-48cc-b14d-d4df74c235f2</t>
+          <t>83a8e2e5-44b5-4571-a0a3-475c6b12e0fe</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -927,34 +987,42 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6170538668", "EffectiveDate": "2026-07-24", "PolicyPaymentInfoList": [{"Amount": "843", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-07-23T17:13:09", "TransactionId": "8cdc2ca9ba9de20f7a76e3a80cfa4d67:d2d6f172ebdac02bbf4eb1516cc2ea94", "TransactionNo": "TGvodE2jEoEeU8"}]}</t>
+          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6170594453", "EffectiveDate": "2026-08-06", "PolicyPaymentInfoList": [{"Amount": "842", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-08-05T20:51:48", "TransactionId": "b3ba14c9d085e75cd3cfeb98885aa337:2a3ab383d5ee752391d877f1cd45c0ac", "TransactionNo": "TM8U8n5eKih6EJ"}]}</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>{"ihub.body": {"consumerAppTransId": "TGvodE2jEoEeU8", "gateway_txn_id": "TGvodE2jEoEeU8", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "843", "payment_id": "8cdc2ca9ba9de20f7a76e3a80cfa4d67:d2d6f172ebdac02bbf4eb1516cc2ea94", "policy_start_date": "2026-07-24", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-07-23 17:13:09"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
+          <t>{"ihub.body": {"consumerAppTransId": "TM8U8n5eKih6EJ", "gateway_txn_id": "TM8U8n5eKih6EJ", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "842", "payment_id": "b3ba14c9d085e75cd3cfeb98885aa337:2a3ab383d5ee752391d877f1cd45c0ac", "policy_start_date": "2026-08-06", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-08-05 20:51:48"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "e307cb73b3f8a8dac25cc9b7a1780771:21758b88e2225ef2bf3d4997bc37a0e4", "encrypted_policy_no": "775d7e19d6a5822f5f1651c68cc7e39b:c6380f382d61a3e25a8fa87018dc30a2", "master_policy": "", "net_premium": 843, "nstp_id": "N500001763548", "nstp_stage": "completed", "payment_id": "036835270dfabb26555d0cf5f53f1af7:908b80ca8d1bf5e95ed8dd77b7a5a0bf", "payment_stage": "completed", "policy_id": "P500192556250", "policy_no": "6170645852-00", "product_id": "M300000000002", "proposal_no": "PR/26/6170538668", "proposal_stage": "completed", "quote_no": "QT/26/6175687549", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Success", "status": 200}</t>
+          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "0876f11e9b406ade765cfdf1bb805cd5:3424cada4ea81d3070054f262565670c", "encrypted_policy_no": "c8888c6171c50861b81223454a04155f:9fd42fe6c2cfc0f9c5833d9fe3c0040d", "master_policy": "", "net_premium": 842, "nstp_id": "N500001850996", "nstp_stage": "completed", "payment_id": "8e08c349984460dac7823c086cd1290d:dfcd786fe4eeecf9f61b706759d041ad", "payment_stage": "completed", "policy_id": "P500197773906", "policy_no": "6170681150-00", "product_id": "M300000000002", "proposal_no": "PR/26/6170594453", "proposal_stage": "completed", "quote_no": "QT/26/6176053802", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>{"ClientRequestId": "62da7d91-33f9-48cc-b14d-d4df74c235f2", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6170645852-00", "CarrierProposalNo": "PR/26/6170538668", "CarrierQuoteRequestId": "QT/26/6175687549", "InspectionId": "N500001763548", "PaymentId": "036835270dfabb26555d0cf5f53f1af7:908b80ca8d1bf5e95ed8dd77b7a5a0bf", "requestId": "P500192556250"}, "ResultCode": 1, "TransactionType": 2003}</t>
+          <t>{"ClientRequestId": "83a8e2e5-44b5-4571-a0a3-475c6b12e0fe", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6170681150-00", "CarrierProposalNo": "PR/26/6170594453", "CarrierQuoteRequestId": "QT/26/6176053802", "InspectionId": "N500001850996", "PaymentId": "8e08c349984460dac7823c086cd1290d:dfcd786fe4eeecf9f61b706759d041ad", "requestId": "P500197773906"}, "ResultCode": 1, "TransactionType": 2003}</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T20:51:49</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-04T23:57:09</t>
+          <t>2026-08-10T23:16:01</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
@@ -962,17 +1030,17 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>6170677969-00</t>
+          <t>6270461067-00</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>0ce36c7d775e8f96d4ceed2a617f9518</t>
+          <t>dede56f7dbe82bd3ac11bc9d37b7b0bc</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>6db2e587-29f8-4264-890d-97d3fd8d2a44</t>
+          <t>3ae3c076-18a6-41ad-b82a-faacea41985c</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -987,34 +1055,42 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6170589741", "EffectiveDate": "2026-08-05", "PolicyPaymentInfoList": [{"Amount": "1374", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-08-04T23:57:08", "TransactionId": "3e93982a459ab3689910ea9fd1e19117:af925455d51084d8172a835b3364b531", "TransactionNo": "TLn6gZDOXDNPga"}]}</t>
+          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6270462763", "EffectiveDate": "2026-08-15", "PolicyPaymentInfoList": [{"Amount": "7602", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-08-10T23:16:00", "TransactionId": "ddfcfbc973885be953997b4616534d98:fe5d85795bf64f41dc0f448f99a5d274", "TransactionNo": "TO9c79dMjGqz0l"}]}</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>{"ihub.body": {"consumerAppTransId": "TLn6gZDOXDNPga", "gateway_txn_id": "TLn6gZDOXDNPga", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "1374", "payment_id": "3e93982a459ab3689910ea9fd1e19117:af925455d51084d8172a835b3364b531", "policy_start_date": "2026-08-05", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-08-04 23:57:08"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
+          <t>{"ihub.body": {"consumerAppTransId": "TO9c79dMjGqz0l", "gateway_txn_id": "TO9c79dMjGqz0l", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "7602", "payment_id": "ddfcfbc973885be953997b4616534d98:fe5d85795bf64f41dc0f448f99a5d274", "policy_start_date": "2026-08-15", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-08-10 23:16:00"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "a138ecac97d25d04f9b697cb90bbd8cd:558503a1be3105fe0865b0a5dd933efa", "encrypted_policy_no": "d64c856525a014021b8819c8921aca5f:5c1e9c90f490b008202d036ed9ca9350", "master_policy": "", "net_premium": 1374, "nstp_id": "N500001843894", "nstp_stage": "completed", "payment_id": "8422f8f1c61551c6512f9b2f5116f92d:221334417c936d8c0d93c8dfce0b8732", "payment_stage": "completed", "policy_id": "P500197370675", "policy_no": "6170677969-00", "product_id": "M300000000002", "proposal_no": "PR/26/6170589741", "proposal_stage": "completed", "quote_no": "QT/26/6176022411", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
+          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "872728eced87e71bfe3c5423c8dd526e:c1b934d15ad5f43d0b41166391dc81e6", "encrypted_policy_no": "2f927c96d97a593dd7f6a9f48ab5507b:4e757484b466e32146326b3f3ef49123", "master_policy": "", "net_premium": 7602, "nstp_id": "N500001884176", "nstp_stage": "completed", "payment_id": "84401574def0b079980a2c16fd428f7a:ade02d07e2d07a7702198ca91beb4cbe", "payment_stage": "completed", "policy_id": "P500199943210", "policy_no": "6270461067-00", "product_id": "M300000000001", "proposal_no": "PR/26/6270462763", "proposal_stage": "completed", "quote_no": "QT/26/6286516113", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>{"ClientRequestId": "6db2e587-29f8-4264-890d-97d3fd8d2a44", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6170677969-00", "CarrierProposalNo": "PR/26/6170589741", "CarrierQuoteRequestId": "QT/26/6176022411", "InspectionId": "N500001843894", "PaymentId": "8422f8f1c61551c6512f9b2f5116f92d:221334417c936d8c0d93c8dfce0b8732", "requestId": "P500197370675"}, "ResultCode": 1, "TransactionType": 2003}</t>
+          <t>{"ClientRequestId": "3ae3c076-18a6-41ad-b82a-faacea41985c", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6270461067-00", "CarrierProposalNo": "PR/26/6270462763", "CarrierQuoteRequestId": "QT/26/6286516113", "InspectionId": "N500001884176", "PaymentId": "84401574def0b079980a2c16fd428f7a:ade02d07e2d07a7702198ca91beb4cbe", "requestId": "P500199943210"}, "ResultCode": 1, "TransactionType": 2003}</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10T23:16:07</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-04T23:57:15</t>
+          <t>2026-08-11T13:27:56</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
@@ -1022,17 +1098,17 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>6170677969-00</t>
+          <t>6270461560-00</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>849e7b02407fd1ae7d0df49854bebd4c</t>
+          <t>18e71bece2bb7a1bec71537d89584ea4</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>cf4c2eff-f45d-4d32-a390-fe28af015b48</t>
+          <t>d1f515f0-2108-4075-9091-276f1ea3463a</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1047,34 +1123,42 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6170589741", "EffectiveDate": "2026-08-05", "PolicyPaymentInfoList": [{"Amount": "1374", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-08-04T23:57:09", "TransactionId": "3e93982a459ab3689910ea9fd1e19117:af925455d51084d8172a835b3364b531", "TransactionNo": "TLn6gZDOXDNPga"}]}</t>
+          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6270462350", "EffectiveDate": "2026-08-10", "PolicyPaymentInfoList": [{"Amount": "7613", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-08-11T13:27:55", "TransactionId": "7966b6bd78538dc1c1a3257bc2e4d0e0:5a3138fb9886b3c4c6b591aed791c493", "TransactionNo": "TO51lI7BZlbcLo"}]}</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>{"ihub.body": {"consumerAppTransId": "TLn6gZDOXDNPga", "gateway_txn_id": "TLn6gZDOXDNPga", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "1374", "payment_id": "3e93982a459ab3689910ea9fd1e19117:af925455d51084d8172a835b3364b531", "policy_start_date": "2026-08-05", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-08-04 23:57:09"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
+          <t>{"ihub.body": {"consumerAppTransId": "TO51lI7BZlbcLo", "gateway_txn_id": "TO51lI7BZlbcLo", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "7613", "payment_id": "7966b6bd78538dc1c1a3257bc2e4d0e0:5a3138fb9886b3c4c6b591aed791c493", "policy_start_date": "2026-08-10", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-08-11 13:27:55"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "31a2bfb01472af1ca788e37826e193e2:cf803dd0d90862a68ce4776ea494505c", "encrypted_policy_no": "7051e7717f1dd23a513c9f730499a90f:b85fb33940d405b9b7a2df6759decabb", "master_policy": "", "net_premium": 1374, "nstp_id": "N500001843894", "nstp_stage": "completed", "payment_id": "fd40b4ee9d80481b2bc9c15260e2e499:84bb9e4c3e262e7cc0e78e97394c65d0", "payment_stage": "completed", "policy_id": "P500197370675", "policy_no": "6170677969-00", "product_id": "M300000000002", "proposal_no": "PR/26/6170589741", "proposal_stage": "completed", "quote_no": "QT/26/6176022411", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Success", "status": 200}</t>
+          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "b50cac7c80bdc034a4d89e9145ff931c:3e65da39f3e4a673b10881143a115f15", "encrypted_policy_no": "4eae3010258a46eee3b48e3b51c2b420:06b4fd70216fe399d22a40f0ad4d7a2d", "master_policy": "", "net_premium": 7613, "nstp_id": "N500001883029", "nstp_stage": "completed", "payment_id": "1756fec825124ee7dac61c189e19eed6:afd855be37be77646c3f217335bede62", "payment_stage": "completed", "policy_id": "P500199875241", "policy_no": "6270461560-00", "product_id": "M300000000001", "proposal_no": "PR/26/6270462350", "proposal_stage": "completed", "quote_no": "QT/26/6286509453", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>{"ClientRequestId": "cf4c2eff-f45d-4d32-a390-fe28af015b48", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6170677969-00", "CarrierProposalNo": "PR/26/6170589741", "CarrierQuoteRequestId": "QT/26/6176022411", "InspectionId": "N500001843894", "PaymentId": "fd40b4ee9d80481b2bc9c15260e2e499:84bb9e4c3e262e7cc0e78e97394c65d0", "requestId": "P500197370675"}, "ResultCode": 1, "TransactionType": 2003}</t>
+          <t>{"ClientRequestId": "d1f515f0-2108-4075-9091-276f1ea3463a", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6270461560-00", "CarrierProposalNo": "PR/26/6270462350", "CarrierQuoteRequestId": "QT/26/6286509453", "InspectionId": "N500001883029", "PaymentId": "1756fec825124ee7dac61c189e19eed6:afd855be37be77646c3f217335bede62", "requestId": "P500199875241"}, "ResultCode": 1, "TransactionType": 2003}</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-11T13:27:56</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05T20:51:49</t>
+          <t>2026-08-15T10:48:31</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
@@ -1082,17 +1166,17 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>6170681150-00</t>
+          <t>6170705588-00</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>ada238190acdde9e08489db376da2ffc</t>
+          <t>e991647d15833a44254a2767f91bc6c1</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>83a8e2e5-44b5-4571-a0a3-475c6b12e0fe</t>
+          <t>b0694ce5-189b-42eb-82d4-970f1d0de6e0</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -1107,34 +1191,42 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6170594453", "EffectiveDate": "2026-08-06", "PolicyPaymentInfoList": [{"Amount": "842", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-08-05T20:51:48", "TransactionId": "b3ba14c9d085e75cd3cfeb98885aa337:2a3ab383d5ee752391d877f1cd45c0ac", "TransactionNo": "TM8U8n5eKih6EJ"}]}</t>
+          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6170634045", "EffectiveDate": "2026-08-16", "PolicyPaymentInfoList": [{"Amount": "843", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-08-15T10:48:30", "TransactionId": "19b07ed7a1e05f20b32f372f1f9683c6:5d168dd74d4f941c7b0d22c86c71018e", "TransactionNo": "TPvYBGUWcRfTGQ"}]}</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>{"ihub.body": {"consumerAppTransId": "TM8U8n5eKih6EJ", "gateway_txn_id": "TM8U8n5eKih6EJ", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "842", "payment_id": "b3ba14c9d085e75cd3cfeb98885aa337:2a3ab383d5ee752391d877f1cd45c0ac", "policy_start_date": "2026-08-06", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-08-05 20:51:48"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
+          <t>{"ihub.body": {"consumerAppTransId": "TPvYBGUWcRfTGQ", "gateway_txn_id": "TPvYBGUWcRfTGQ", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "843", "payment_id": "19b07ed7a1e05f20b32f372f1f9683c6:5d168dd74d4f941c7b0d22c86c71018e", "policy_start_date": "2026-08-16", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-08-15 10:48:30"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "0876f11e9b406ade765cfdf1bb805cd5:3424cada4ea81d3070054f262565670c", "encrypted_policy_no": "c8888c6171c50861b81223454a04155f:9fd42fe6c2cfc0f9c5833d9fe3c0040d", "master_policy": "", "net_premium": 842, "nstp_id": "N500001850996", "nstp_stage": "completed", "payment_id": "8e08c349984460dac7823c086cd1290d:dfcd786fe4eeecf9f61b706759d041ad", "payment_stage": "completed", "policy_id": "P500197773906", "policy_no": "6170681150-00", "product_id": "M300000000002", "proposal_no": "PR/26/6170594453", "proposal_stage": "completed", "quote_no": "QT/26/6176053802", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
+          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "eb1a24073daf4c46acce07f3ecf915a2:ec9335d88ff3d6088d1ad1928f3941da", "encrypted_policy_no": "92f017554c80e4f1209958d58453b2b4:7ec66e75fc75d131c881a04deeb09ae9", "master_policy": "", "net_premium": 843, "nstp_id": "N500001913499", "nstp_stage": "completed", "payment_id": "8f4e6605556908eaaa7c94e4b842227d:bd76a6ab65ea03dd55b836acb7b82662", "payment_stage": "completed", "policy_id": "P500201743983", "policy_no": "6170705588-00", "product_id": "M300000000002", "proposal_no": "PR/26/6170634045", "proposal_stage": "completed", "quote_no": "QT/26/6176326937", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Success", "status": 200}</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>{"ClientRequestId": "83a8e2e5-44b5-4571-a0a3-475c6b12e0fe", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6170681150-00", "CarrierProposalNo": "PR/26/6170594453", "CarrierQuoteRequestId": "QT/26/6176053802", "InspectionId": "N500001850996", "PaymentId": "8e08c349984460dac7823c086cd1290d:dfcd786fe4eeecf9f61b706759d041ad", "requestId": "P500197773906"}, "ResultCode": 1, "TransactionType": 2003}</t>
+          <t>{"ClientRequestId": "b0694ce5-189b-42eb-82d4-970f1d0de6e0", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6170705588-00", "CarrierProposalNo": "PR/26/6170634045", "CarrierQuoteRequestId": "QT/26/6176326937", "InspectionId": "N500001913499", "PaymentId": "8f4e6605556908eaaa7c94e4b842227d:bd76a6ab65ea03dd55b836acb7b82662", "requestId": "P500201743983"}, "ResultCode": 1, "TransactionType": 2003}</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-15T10:48:31</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10T23:16:01</t>
+          <t>2026-08-15T11:20:13</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
@@ -1142,17 +1234,17 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>6270461067-00</t>
+          <t>6270466181-00</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>dede56f7dbe82bd3ac11bc9d37b7b0bc</t>
+          <t>595a9e7303852f1a28a96c03595b0029</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>3ae3c076-18a6-41ad-b82a-faacea41985c</t>
+          <t>1e664a00-aecc-414a-82a9-cae94ad02ef3</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1167,34 +1259,42 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6270462763", "EffectiveDate": "2026-08-15", "PolicyPaymentInfoList": [{"Amount": "7602", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-08-10T23:16:00", "TransactionId": "ddfcfbc973885be953997b4616534d98:fe5d85795bf64f41dc0f448f99a5d274", "TransactionNo": "TO9c79dMjGqz0l"}]}</t>
+          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6270471733", "EffectiveDate": "2026-08-16", "PolicyPaymentInfoList": [{"Amount": "2913", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-08-15T11:20:12", "TransactionId": "93ee2494ea2c733a2eee5567253323cc:f3a3f3935a08605b0563289a0de4a4a0", "TransactionNo": "TPw5ghl5raw4FB"}]}</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>{"ihub.body": {"consumerAppTransId": "TO9c79dMjGqz0l", "gateway_txn_id": "TO9c79dMjGqz0l", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "7602", "payment_id": "ddfcfbc973885be953997b4616534d98:fe5d85795bf64f41dc0f448f99a5d274", "policy_start_date": "2026-08-15", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-08-10 23:16:00"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
+          <t>{"ihub.body": {"consumerAppTransId": "TPw5ghl5raw4FB", "gateway_txn_id": "TPw5ghl5raw4FB", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "2913", "payment_id": "93ee2494ea2c733a2eee5567253323cc:f3a3f3935a08605b0563289a0de4a4a0", "policy_start_date": "2026-08-16", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-08-15 11:20:12"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "872728eced87e71bfe3c5423c8dd526e:c1b934d15ad5f43d0b41166391dc81e6", "encrypted_policy_no": "2f927c96d97a593dd7f6a9f48ab5507b:4e757484b466e32146326b3f3ef49123", "master_policy": "", "net_premium": 7602, "nstp_id": "N500001884176", "nstp_stage": "completed", "payment_id": "84401574def0b079980a2c16fd428f7a:ade02d07e2d07a7702198ca91beb4cbe", "payment_stage": "completed", "policy_id": "P500199943210", "policy_no": "6270461067-00", "product_id": "M300000000001", "proposal_no": "PR/26/6270462763", "proposal_stage": "completed", "quote_no": "QT/26/6286516113", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
+          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "bd842210f6c748668b7d6bdfb520efa1:211d56ced6785e50905c0aa3b19b52d4", "encrypted_policy_no": "e85ed9c40886935ce1c391f5058ed71b:7f301c8b2c529ba04f577dc93c695288", "master_policy": "", "net_premium": 2913, "nstp_id": "N500001913651", "nstp_stage": "completed", "payment_id": "e5e7a58213052ba5cc7c3e3fd88ed9bb:1e1f51d04959697ea49181e9cbaec4ba", "payment_stage": "completed", "policy_id": "P500201754993", "policy_no": "6270466181-00", "product_id": "M300000000001", "proposal_no": "PR/26/6270471733", "proposal_stage": "completed", "quote_no": "QT/26/6286816723", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>{"ClientRequestId": "3ae3c076-18a6-41ad-b82a-faacea41985c", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6270461067-00", "CarrierProposalNo": "PR/26/6270462763", "CarrierQuoteRequestId": "QT/26/6286516113", "InspectionId": "N500001884176", "PaymentId": "84401574def0b079980a2c16fd428f7a:ade02d07e2d07a7702198ca91beb4cbe", "requestId": "P500199943210"}, "ResultCode": 1, "TransactionType": 2003}</t>
+          <t>{"ClientRequestId": "1e664a00-aecc-414a-82a9-cae94ad02ef3", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6270466181-00", "CarrierProposalNo": "PR/26/6270471733", "CarrierQuoteRequestId": "QT/26/6286816723", "InspectionId": "N500001913651", "PaymentId": "e5e7a58213052ba5cc7c3e3fd88ed9bb:1e1f51d04959697ea49181e9cbaec4ba", "requestId": "P500201754993"}, "ResultCode": 1, "TransactionType": 2003}</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-15T11:20:13</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10T23:16:07</t>
+          <t>2026-08-18T07:21:58</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
@@ -1202,17 +1302,17 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>6270461067-00</t>
+          <t>6170711333-00</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>d4ebac443b71d7ad07f0a5dcc3b186e2</t>
+          <t>8eee38ce1a60968de13180cf354698c3</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>f4aec3c2-665d-427c-996f-1165b58b6b1a</t>
+          <t>1e0e2c49-d6c3-4b67-81ba-1e9341f62d22</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -1227,34 +1327,42 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6270462763", "EffectiveDate": "2026-08-15", "PolicyPaymentInfoList": [{"Amount": "7602", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-08-10T23:16:06", "TransactionId": "ddfcfbc973885be953997b4616534d98:fe5d85795bf64f41dc0f448f99a5d274", "TransactionNo": "TO9c79dMjGqz0l"}]}</t>
+          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6170642192", "EffectiveDate": "2026-08-19", "PolicyPaymentInfoList": [{"Amount": "843", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-08-18T07:21:58", "TransactionId": "6c94a60673b2c57d8e982ac26f893e42:9afb91da2e5fa69f5bcf37ff9d56a71b", "TransactionNo": "TR3dTPLtZecico"}]}</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>{"ihub.body": {"consumerAppTransId": "TO9c79dMjGqz0l", "gateway_txn_id": "TO9c79dMjGqz0l", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "7602", "payment_id": "ddfcfbc973885be953997b4616534d98:fe5d85795bf64f41dc0f448f99a5d274", "policy_start_date": "2026-08-15", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-08-10 23:16:06"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
+          <t>{"ihub.body": {"consumerAppTransId": "TR3dTPLtZecico", "gateway_txn_id": "TR3dTPLtZecico", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "843", "payment_id": "6c94a60673b2c57d8e982ac26f893e42:9afb91da2e5fa69f5bcf37ff9d56a71b", "policy_start_date": "2026-08-19", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-08-18 07:21:58"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "d7cfcc666274209ab4a425db032f8ab0:d452fe732f20241f68917f58acd03518", "encrypted_policy_no": "ca4907dcfc078ca82380b6e2e0f5a819:46f72a894135f7b17d9f4ca4f1ba33d9", "master_policy": "", "net_premium": 7602, "nstp_id": "N500001884176", "nstp_stage": "completed", "payment_id": "5a507294b3bf637f1d146dd814a6f947:4021f164637b0584195e177395bffa5b", "payment_stage": "completed", "policy_id": "P500199943210", "policy_no": "6270461067-00", "product_id": "M300000000001", "proposal_no": "PR/26/6270462763", "proposal_stage": "completed", "quote_no": "QT/26/6286516113", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Success", "status": 200}</t>
+          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "78aad56e62d6b875d5d881789f2f9560:2be575371c0f9b89b2c02b79834153db", "encrypted_policy_no": "e17dd112f12127242fdf7e98cbdef125:c767f330d70e94221e94d1247dbbbc91", "master_policy": "", "net_premium": 843, "nstp_id": "N500001928299", "nstp_stage": "completed", "payment_id": "45613000657dde3a9f4a880b2330ef8a:f3fa2c2645c361e3f066f37374ce28ae", "payment_stage": "completed", "policy_id": "P500202769169", "policy_no": "6170711333-00", "product_id": "M300000000002", "proposal_no": "PR/26/6170642192", "proposal_stage": "completed", "quote_no": "QT/26/6176391054", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>{"ClientRequestId": "f4aec3c2-665d-427c-996f-1165b58b6b1a", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6270461067-00", "CarrierProposalNo": "PR/26/6270462763", "CarrierQuoteRequestId": "QT/26/6286516113", "InspectionId": "N500001884176", "PaymentId": "5a507294b3bf637f1d146dd814a6f947:4021f164637b0584195e177395bffa5b", "requestId": "P500199943210"}, "ResultCode": 1, "TransactionType": 2003}</t>
+          <t>{"ClientRequestId": "1e0e2c49-d6c3-4b67-81ba-1e9341f62d22", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6170711333-00", "CarrierProposalNo": "PR/26/6170642192", "CarrierQuoteRequestId": "QT/26/6176391054", "InspectionId": "N500001928299", "PaymentId": "45613000657dde3a9f4a880b2330ef8a:f3fa2c2645c361e3f066f37374ce28ae", "requestId": "P500202769169"}, "ResultCode": 1, "TransactionType": 2003}</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-18T07:21:58</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11T13:27:56</t>
+          <t>2026-08-21T10:34:20</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -1262,17 +1370,17 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>6270461560-00</t>
+          <t>6170719551-00</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>18e71bece2bb7a1bec71537d89584ea4</t>
+          <t>fc9e2493feeb39330b499198a8e626ac</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>d1f515f0-2108-4075-9091-276f1ea3463a</t>
+          <t>f8639e2c-23e1-437b-8993-ff4658e1de37</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1287,34 +1395,42 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6270462350", "EffectiveDate": "2026-08-10", "PolicyPaymentInfoList": [{"Amount": "7613", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-08-11T13:27:55", "TransactionId": "7966b6bd78538dc1c1a3257bc2e4d0e0:5a3138fb9886b3c4c6b591aed791c493", "TransactionNo": "TO51lI7BZlbcLo"}]}</t>
+          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6170656853", "EffectiveDate": "2026-08-21", "PolicyPaymentInfoList": [{"Amount": "893", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-08-21T10:34:20", "TransactionId": "c427a91f67ca2fa767df02b2bda78cc0:520346e774c87f1ddd061f9470830179", "TransactionNo": "TSIVrrpGnruz8L"}]}</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>{"ihub.body": {"consumerAppTransId": "TO51lI7BZlbcLo", "gateway_txn_id": "TO51lI7BZlbcLo", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "7613", "payment_id": "7966b6bd78538dc1c1a3257bc2e4d0e0:5a3138fb9886b3c4c6b591aed791c493", "policy_start_date": "2026-08-10", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-08-11 13:27:55"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
+          <t>{"ihub.body": {"consumerAppTransId": "TSIVrrpGnruz8L", "gateway_txn_id": "TSIVrrpGnruz8L", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "893", "payment_id": "c427a91f67ca2fa767df02b2bda78cc0:520346e774c87f1ddd061f9470830179", "policy_start_date": "2026-08-21", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-08-21 10:34:20"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "b50cac7c80bdc034a4d89e9145ff931c:3e65da39f3e4a673b10881143a115f15", "encrypted_policy_no": "4eae3010258a46eee3b48e3b51c2b420:06b4fd70216fe399d22a40f0ad4d7a2d", "master_policy": "", "net_premium": 7613, "nstp_id": "N500001883029", "nstp_stage": "completed", "payment_id": "1756fec825124ee7dac61c189e19eed6:afd855be37be77646c3f217335bede62", "payment_stage": "completed", "policy_id": "P500199875241", "policy_no": "6270461560-00", "product_id": "M300000000001", "proposal_no": "PR/26/6270462350", "proposal_stage": "completed", "quote_no": "QT/26/6286509453", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
+          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "00ca135c22db583999fe446c48a853ca:6f6cb850c17ef59d01b8da655b6e005e", "encrypted_policy_no": "3f693ac2a76851353d938a93dadc46d7:cbd65153bb35a314275141a54241ae4e", "master_policy": "", "net_premium": 893, "nstp_id": "N500001950940", "nstp_stage": "completed", "payment_id": "484bb5122e43e5726e34368db0f61033:80d46ca07d49687584bb2cb2431ed78e", "payment_stage": "completed", "policy_id": "P500204183574", "policy_no": "6170719551-00", "product_id": "M300000000002", "proposal_no": "PR/26/6170656853", "proposal_stage": "completed", "quote_no": "QT/26/6176484797", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>{"ClientRequestId": "d1f515f0-2108-4075-9091-276f1ea3463a", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6270461560-00", "CarrierProposalNo": "PR/26/6270462350", "CarrierQuoteRequestId": "QT/26/6286509453", "InspectionId": "N500001883029", "PaymentId": "1756fec825124ee7dac61c189e19eed6:afd855be37be77646c3f217335bede62", "requestId": "P500199875241"}, "ResultCode": 1, "TransactionType": 2003}</t>
+          <t>{"ClientRequestId": "f8639e2c-23e1-437b-8993-ff4658e1de37", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6170719551-00", "CarrierProposalNo": "PR/26/6170656853", "CarrierQuoteRequestId": "QT/26/6176484797", "InspectionId": "N500001950940", "PaymentId": "484bb5122e43e5726e34368db0f61033:80d46ca07d49687584bb2cb2431ed78e", "requestId": "P500204183574"}, "ResultCode": 1, "TransactionType": 2003}</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T10:34:22</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15T10:48:31</t>
+          <t>2026-08-23T18:54:09</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -1322,17 +1438,17 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>6170705588-00</t>
+          <t>6170725329-00</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>e991647d15833a44254a2767f91bc6c1</t>
+          <t>60a059df8fcebe0a020e55affbfd87a5</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>b0694ce5-189b-42eb-82d4-970f1d0de6e0</t>
+          <t>437c430b-2785-432b-bf7e-f96c458512a9</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -1347,34 +1463,42 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6170634045", "EffectiveDate": "2026-08-16", "PolicyPaymentInfoList": [{"Amount": "843", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-08-15T10:48:30", "TransactionId": "19b07ed7a1e05f20b32f372f1f9683c6:5d168dd74d4f941c7b0d22c86c71018e", "TransactionNo": "TPvYBGUWcRfTGQ"}]}</t>
+          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6170666328", "EffectiveDate": "2026-08-24", "PolicyPaymentInfoList": [{"Amount": "842", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-08-23T18:54:08", "TransactionId": "d4600d2da057a3e40340994d216ec15d:c5cd422c5142d6df20625b4bb9ff328d", "TransactionNo": "TTE64rmCQep66E"}]}</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>{"ihub.body": {"consumerAppTransId": "TPvYBGUWcRfTGQ", "gateway_txn_id": "TPvYBGUWcRfTGQ", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "843", "payment_id": "19b07ed7a1e05f20b32f372f1f9683c6:5d168dd74d4f941c7b0d22c86c71018e", "policy_start_date": "2026-08-16", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-08-15 10:48:30"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
+          <t>{"ihub.body": {"consumerAppTransId": "TTE64rmCQep66E", "gateway_txn_id": "TTE64rmCQep66E", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "842", "payment_id": "d4600d2da057a3e40340994d216ec15d:c5cd422c5142d6df20625b4bb9ff328d", "policy_start_date": "2026-08-24", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-08-23 18:54:08"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "eb1a24073daf4c46acce07f3ecf915a2:ec9335d88ff3d6088d1ad1928f3941da", "encrypted_policy_no": "92f017554c80e4f1209958d58453b2b4:7ec66e75fc75d131c881a04deeb09ae9", "master_policy": "", "net_premium": 843, "nstp_id": "N500001913499", "nstp_stage": "completed", "payment_id": "8f4e6605556908eaaa7c94e4b842227d:bd76a6ab65ea03dd55b836acb7b82662", "payment_stage": "completed", "policy_id": "P500201743983", "policy_no": "6170705588-00", "product_id": "M300000000002", "proposal_no": "PR/26/6170634045", "proposal_stage": "completed", "quote_no": "QT/26/6176326937", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Success", "status": 200}</t>
+          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "46c2f22cf5e9bbf328dc1cad0f064168:0bc7700ef571439cbf8645756c43f50f", "encrypted_policy_no": "772ef6e6b773d384ed8ba91c7139adf2:f7e1947dfc0303ed6a9211f3534e4b70", "master_policy": "", "net_premium": 842, "nstp_id": "N500001966970", "nstp_stage": "completed", "payment_id": "cda8b648ef0005b78a67ca5eff45f369:be4b478a2a977f9dab08281d4ff52ec9", "payment_stage": "completed", "policy_id": "P500205258244", "policy_no": "6170725329-00", "product_id": "M300000000002", "proposal_no": "PR/26/6170666328", "proposal_stage": "completed", "quote_no": "QT/26/6176550842", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>{"ClientRequestId": "b0694ce5-189b-42eb-82d4-970f1d0de6e0", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6170705588-00", "CarrierProposalNo": "PR/26/6170634045", "CarrierQuoteRequestId": "QT/26/6176326937", "InspectionId": "N500001913499", "PaymentId": "8f4e6605556908eaaa7c94e4b842227d:bd76a6ab65ea03dd55b836acb7b82662", "requestId": "P500201743983"}, "ResultCode": 1, "TransactionType": 2003}</t>
+          <t>{"ClientRequestId": "437c430b-2785-432b-bf7e-f96c458512a9", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6170725329-00", "CarrierProposalNo": "PR/26/6170666328", "CarrierQuoteRequestId": "QT/26/6176550842", "InspectionId": "N500001966970", "PaymentId": "cda8b648ef0005b78a67ca5eff45f369:be4b478a2a977f9dab08281d4ff52ec9", "requestId": "P500205258244"}, "ResultCode": 1, "TransactionType": 2003}</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-23T18:54:09</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15T10:48:31</t>
+          <t>2026-08-26T10:35:44</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -1382,17 +1506,17 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>6170705588-00</t>
+          <t>6270479230-00</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>112d7033a79748f7b8c686561ff516fd</t>
+          <t>515b7101c3e0e0a55571c0a407b51533</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>8611f555-23f4-42b9-867f-f9981fc8b753</t>
+          <t>6b083cdc-67bd-4a1f-8905-96a696ca3c6b</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -1407,34 +1531,42 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6170634045", "EffectiveDate": "2026-08-16", "PolicyPaymentInfoList": [{"Amount": "843", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-08-15T10:48:30", "TransactionId": "19b07ed7a1e05f20b32f372f1f9683c6:5d168dd74d4f941c7b0d22c86c71018e", "TransactionNo": "TPvYBGUWcRfTGQ"}]}</t>
+          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6270495617", "EffectiveDate": "2026-09-02", "PolicyPaymentInfoList": [{"Amount": "8367", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-08-26T10:35:43", "TransactionId": "242b54330fd1c4db260cc8ec72936dde:8dbf8f8c09f4d4a7d21a659aecc326f3", "TransactionNo": "TUHCwfpI0VAVxC"}]}</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>{"ihub.body": {"consumerAppTransId": "TPvYBGUWcRfTGQ", "gateway_txn_id": "TPvYBGUWcRfTGQ", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "843", "payment_id": "19b07ed7a1e05f20b32f372f1f9683c6:5d168dd74d4f941c7b0d22c86c71018e", "policy_start_date": "2026-08-16", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-08-15 10:48:30"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
+          <t>{"ihub.body": {"consumerAppTransId": "TUHCwfpI0VAVxC", "gateway_txn_id": "TUHCwfpI0VAVxC", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "8367", "payment_id": "242b54330fd1c4db260cc8ec72936dde:8dbf8f8c09f4d4a7d21a659aecc326f3", "policy_start_date": "2026-09-02", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-08-26 10:35:43"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "31c1f8d64a7d17dfc2ba2fa494163377:410f216f4889a9e51eac4b115367615b", "encrypted_policy_no": "1b85968ae8ace53fea877ef5fd670d50:5cf9b0a8fe515c79dd322e20e5e5183d", "master_policy": "", "net_premium": 843, "nstp_id": "N500001913499", "nstp_stage": "completed", "payment_id": "d01517165df14bf4354f6dcfcceea9cb:e137c59c757eb9aa972d74ca0e46b03c", "payment_stage": "completed", "policy_id": "P500201743983", "policy_no": "6170705588-00", "product_id": "M300000000002", "proposal_no": "PR/26/6170634045", "proposal_stage": "completed", "quote_no": "QT/26/6176326937", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
+          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "d1d56bfda9ff92498d28047dfaadbba3:c5857debffbb2d2951df9bd221a100d5", "encrypted_policy_no": "5582bf7528d6f4a7e29a7f5f84b1c2a5:ed73e1c599ba3999879f10e120586999", "master_policy": "", "net_premium": 8367, "nstp_id": "N500001983446", "nstp_stage": "completed", "payment_id": "30beee7616b8dafb65cbf1c79e6a2aa5:c1328db2403f3db3eeaf22021825a571", "payment_stage": "completed", "policy_id": "P500206383696", "policy_no": "6270479230-00", "product_id": "M300000000001", "proposal_no": "PR/26/6270495617", "proposal_stage": "completed", "quote_no": "QT/26/6287576616", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>{"ClientRequestId": "8611f555-23f4-42b9-867f-f9981fc8b753", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6170705588-00", "CarrierProposalNo": "PR/26/6170634045", "CarrierQuoteRequestId": "QT/26/6176326937", "InspectionId": "N500001913499", "PaymentId": "d01517165df14bf4354f6dcfcceea9cb:e137c59c757eb9aa972d74ca0e46b03c", "requestId": "P500201743983"}, "ResultCode": 1, "TransactionType": 2003}</t>
+          <t>{"ClientRequestId": "6b083cdc-67bd-4a1f-8905-96a696ca3c6b", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6270479230-00", "CarrierProposalNo": "PR/26/6270495617", "CarrierQuoteRequestId": "QT/26/6287576616", "InspectionId": "N500001983446", "PaymentId": "30beee7616b8dafb65cbf1c79e6a2aa5:c1328db2403f3db3eeaf22021825a571", "requestId": "P500206383696"}, "ResultCode": 1, "TransactionType": 2003}</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26T10:35:45</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15T11:20:13</t>
+          <t>2026-08-31T20:37:04</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -1442,17 +1574,17 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>6270466181-00</t>
+          <t>6170743506-00</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>595a9e7303852f1a28a96c03595b0029</t>
+          <t>d9fbbfaeefd5d4334975b3b277229adb</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>1e664a00-aecc-414a-82a9-cae94ad02ef3</t>
+          <t>f23871d4-ec7c-4c9c-a87c-70461144ac55</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -1467,34 +1599,42 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6270471733", "EffectiveDate": "2026-08-16", "PolicyPaymentInfoList": [{"Amount": "2913", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-08-15T11:20:12", "TransactionId": "93ee2494ea2c733a2eee5567253323cc:f3a3f3935a08605b0563289a0de4a4a0", "TransactionNo": "TPw5ghl5raw4FB"}]}</t>
+          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6170701071", "EffectiveDate": "2026-09-01", "PolicyPaymentInfoList": [{"Amount": "1285", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-08-31T20:37:03", "TransactionId": "d4abc8259e09ee9f4b2591a083cf720c:adf5184d95b9d62eb21cff3bac25182e", "TransactionNo": "TWQ7vcNMkcMtIL"}]}</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>{"ihub.body": {"consumerAppTransId": "TPw5ghl5raw4FB", "gateway_txn_id": "TPw5ghl5raw4FB", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "2913", "payment_id": "93ee2494ea2c733a2eee5567253323cc:f3a3f3935a08605b0563289a0de4a4a0", "policy_start_date": "2026-08-16", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-08-15 11:20:12"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
+          <t>{"ihub.body": {"consumerAppTransId": "TWQ7vcNMkcMtIL", "gateway_txn_id": "TWQ7vcNMkcMtIL", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "1285", "payment_id": "d4abc8259e09ee9f4b2591a083cf720c:adf5184d95b9d62eb21cff3bac25182e", "policy_start_date": "2026-09-01", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-08-31 20:37:03"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "bd842210f6c748668b7d6bdfb520efa1:211d56ced6785e50905c0aa3b19b52d4", "encrypted_policy_no": "e85ed9c40886935ce1c391f5058ed71b:7f301c8b2c529ba04f577dc93c695288", "master_policy": "", "net_premium": 2913, "nstp_id": "N500001913651", "nstp_stage": "completed", "payment_id": "e5e7a58213052ba5cc7c3e3fd88ed9bb:1e1f51d04959697ea49181e9cbaec4ba", "payment_stage": "completed", "policy_id": "P500201754993", "policy_no": "6270466181-00", "product_id": "M300000000001", "proposal_no": "PR/26/6270471733", "proposal_stage": "completed", "quote_no": "QT/26/6286816723", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
+          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "ddd99c20a764e8ac0a07bca010c22021:14c214413eb50bbb7e9d831ee5e6df5a", "encrypted_policy_no": "c592381ad71e0b4d1956f30dff984aee:b1fc13ef179c008f1bb016d30c0a28ad", "master_policy": "", "net_premium": 1285, "nstp_id": "N500002021467", "nstp_stage": "completed", "payment_id": "afb898ed25b77e8c5edf008a91f5cb4f:6ae4e65047f0c160d3d98501e70f3058", "payment_stage": "completed", "policy_id": "P500209010887", "policy_no": "6170743506-00", "product_id": "M300000000002", "proposal_no": "PR/26/6170701071", "proposal_stage": "completed", "quote_no": "QT/26/6176761122", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>{"ClientRequestId": "1e664a00-aecc-414a-82a9-cae94ad02ef3", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6270466181-00", "CarrierProposalNo": "PR/26/6270471733", "CarrierQuoteRequestId": "QT/26/6286816723", "InspectionId": "N500001913651", "PaymentId": "e5e7a58213052ba5cc7c3e3fd88ed9bb:1e1f51d04959697ea49181e9cbaec4ba", "requestId": "P500201754993"}, "ResultCode": 1, "TransactionType": 2003}</t>
+          <t>{"ClientRequestId": "f23871d4-ec7c-4c9c-a87c-70461144ac55", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6170743506-00", "CarrierProposalNo": "PR/26/6170701071", "CarrierQuoteRequestId": "QT/26/6176761122", "InspectionId": "N500002021467", "PaymentId": "afb898ed25b77e8c5edf008a91f5cb4f:6ae4e65047f0c160d3d98501e70f3058", "requestId": "P500209010887"}, "ResultCode": 1, "TransactionType": 2003}</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31T20:37:06</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18T07:21:58</t>
+          <t>2026-09-02T04:13:05</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -1502,17 +1642,17 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>6170711333-00</t>
+          <t>6170746652-00</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>8eee38ce1a60968de13180cf354698c3</t>
+          <t>5a9555ac25de494af5adadb738cdab49</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>1e0e2c49-d6c3-4b67-81ba-1e9341f62d22</t>
+          <t>355bf614-8c68-4f8a-804b-6f2ed1505db1</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -1527,34 +1667,42 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6170642192", "EffectiveDate": "2026-08-19", "PolicyPaymentInfoList": [{"Amount": "843", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-08-18T07:21:58", "TransactionId": "6c94a60673b2c57d8e982ac26f893e42:9afb91da2e5fa69f5bcf37ff9d56a71b", "TransactionNo": "TR3dTPLtZecico"}]}</t>
+          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6170706695", "EffectiveDate": "2026-09-03", "PolicyPaymentInfoList": [{"Amount": "1374", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-09-02T04:13:04", "TransactionId": "45a72cc153b5f202b926b37119a4de45:026f6dd545f62a770eb1b2d58a3eb37d", "TransactionNo": "TWwQXfsLqZhlas"}]}</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>{"ihub.body": {"consumerAppTransId": "TR3dTPLtZecico", "gateway_txn_id": "TR3dTPLtZecico", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "843", "payment_id": "6c94a60673b2c57d8e982ac26f893e42:9afb91da2e5fa69f5bcf37ff9d56a71b", "policy_start_date": "2026-08-19", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-08-18 07:21:58"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
+          <t>{"ihub.body": {"consumerAppTransId": "TWwQXfsLqZhlas", "gateway_txn_id": "TWwQXfsLqZhlas", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "1374", "payment_id": "45a72cc153b5f202b926b37119a4de45:026f6dd545f62a770eb1b2d58a3eb37d", "policy_start_date": "2026-09-03", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-09-02 04:13:04"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "78aad56e62d6b875d5d881789f2f9560:2be575371c0f9b89b2c02b79834153db", "encrypted_policy_no": "e17dd112f12127242fdf7e98cbdef125:c767f330d70e94221e94d1247dbbbc91", "master_policy": "", "net_premium": 843, "nstp_id": "N500001928299", "nstp_stage": "completed", "payment_id": "45613000657dde3a9f4a880b2330ef8a:f3fa2c2645c361e3f066f37374ce28ae", "payment_stage": "completed", "policy_id": "P500202769169", "policy_no": "6170711333-00", "product_id": "M300000000002", "proposal_no": "PR/26/6170642192", "proposal_stage": "completed", "quote_no": "QT/26/6176391054", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
+          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "02b9a27d0c4d5990caf6b64c58b7f121:40d017d5f41614a76329f00884b7a9fa", "encrypted_policy_no": "17e32c558a1c4a9c8eb7f6d1b7662a82:b3835c140178c5c192b59f5d145ee344", "master_policy": "", "net_premium": 1374, "nstp_id": "N500002029991", "nstp_stage": "completed", "payment_id": "dadf53813b5f1be63dd0c32803d3ec67:8ed8a861e045e35058a141e6ee691965", "payment_stage": "completed", "policy_id": "P500209687513", "policy_no": "6170746652-00", "product_id": "M300000000002", "proposal_no": "PR/26/6170706695", "proposal_stage": "completed", "quote_no": "QT/26/6176796168", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>{"ClientRequestId": "1e0e2c49-d6c3-4b67-81ba-1e9341f62d22", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6170711333-00", "CarrierProposalNo": "PR/26/6170642192", "CarrierQuoteRequestId": "QT/26/6176391054", "InspectionId": "N500001928299", "PaymentId": "45613000657dde3a9f4a880b2330ef8a:f3fa2c2645c361e3f066f37374ce28ae", "requestId": "P500202769169"}, "ResultCode": 1, "TransactionType": 2003}</t>
+          <t>{"ClientRequestId": "355bf614-8c68-4f8a-804b-6f2ed1505db1", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6170746652-00", "CarrierProposalNo": "PR/26/6170706695", "CarrierQuoteRequestId": "QT/26/6176796168", "InspectionId": "N500002029991", "PaymentId": "dadf53813b5f1be63dd0c32803d3ec67:8ed8a861e045e35058a141e6ee691965", "requestId": "P500209687513"}, "ResultCode": 1, "TransactionType": 2003}</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02T04:13:06</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21T10:34:20</t>
+          <t>2026-09-02T15:54:22</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -1562,17 +1710,17 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>6170719551-00</t>
+          <t>6170748395-00</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>fc9e2493feeb39330b499198a8e626ac</t>
+          <t>ea722230d5dea0c06b03978d1350556c</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>f8639e2c-23e1-437b-8993-ff4658e1de37</t>
+          <t>b07934b8-dca3-48a6-88b8-6cb870adb157</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -1587,34 +1735,42 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6170656853", "EffectiveDate": "2026-08-21", "PolicyPaymentInfoList": [{"Amount": "893", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-08-21T10:34:20", "TransactionId": "c427a91f67ca2fa767df02b2bda78cc0:520346e774c87f1ddd061f9470830179", "TransactionNo": "TSIVrrpGnruz8L"}]}</t>
+          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6170710217", "EffectiveDate": "2026-09-03", "PolicyPaymentInfoList": [{"Amount": "843", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-09-02T15:54:21", "TransactionId": "63dc00f0a7a0b038fb239d8af346dc1a:bff2effcd009a9b2c1e0747857aa2bd6", "TransactionNo": "TX8NHVzZdTLOoz"}]}</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>{"ihub.body": {"consumerAppTransId": "TSIVrrpGnruz8L", "gateway_txn_id": "TSIVrrpGnruz8L", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "893", "payment_id": "c427a91f67ca2fa767df02b2bda78cc0:520346e774c87f1ddd061f9470830179", "policy_start_date": "2026-08-21", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-08-21 10:34:20"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
+          <t>{"ihub.body": {"consumerAppTransId": "TX8NHVzZdTLOoz", "gateway_txn_id": "TX8NHVzZdTLOoz", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "843", "payment_id": "63dc00f0a7a0b038fb239d8af346dc1a:bff2effcd009a9b2c1e0747857aa2bd6", "policy_start_date": "2026-09-03", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-09-02 15:54:21"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "00ca135c22db583999fe446c48a853ca:6f6cb850c17ef59d01b8da655b6e005e", "encrypted_policy_no": "3f693ac2a76851353d938a93dadc46d7:cbd65153bb35a314275141a54241ae4e", "master_policy": "", "net_premium": 893, "nstp_id": "N500001950940", "nstp_stage": "completed", "payment_id": "484bb5122e43e5726e34368db0f61033:80d46ca07d49687584bb2cb2431ed78e", "payment_stage": "completed", "policy_id": "P500204183574", "policy_no": "6170719551-00", "product_id": "M300000000002", "proposal_no": "PR/26/6170656853", "proposal_stage": "completed", "quote_no": "QT/26/6176484797", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
+          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "f883b4121427000b1a474f874343e7c9:af0986d46ed85850b236bae29738d6f9", "encrypted_policy_no": "0ba2a8306f35c3ff6a24c5b1bde6c2ff:0463ee2ed44e76183b8f06509043c497", "master_policy": "", "net_premium": 843, "nstp_id": "N500002035031", "nstp_stage": "completed", "payment_id": "43b9cf968f756b3023d48605cc8aba49:e8a5c497444a2e0edc43f533a611356b", "payment_stage": "completed", "policy_id": "P500209987686", "policy_no": "6170748395-00", "product_id": "M300000000002", "proposal_no": "PR/26/6170710217", "proposal_stage": "completed", "quote_no": "QT/26/6176815685", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>{"ClientRequestId": "f8639e2c-23e1-437b-8993-ff4658e1de37", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6170719551-00", "CarrierProposalNo": "PR/26/6170656853", "CarrierQuoteRequestId": "QT/26/6176484797", "InspectionId": "N500001950940", "PaymentId": "484bb5122e43e5726e34368db0f61033:80d46ca07d49687584bb2cb2431ed78e", "requestId": "P500204183574"}, "ResultCode": 1, "TransactionType": 2003}</t>
+          <t>{"ClientRequestId": "b07934b8-dca3-48a6-88b8-6cb870adb157", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6170748395-00", "CarrierProposalNo": "PR/26/6170710217", "CarrierQuoteRequestId": "QT/26/6176815685", "InspectionId": "N500002035031", "PaymentId": "43b9cf968f756b3023d48605cc8aba49:e8a5c497444a2e0edc43f533a611356b", "requestId": "P500209987686"}, "ResultCode": 1, "TransactionType": 2003}</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02T15:54:23</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21T10:34:22</t>
+          <t>2026-09-06T09:43:29</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -1622,17 +1778,17 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>6170719551-00</t>
+          <t>6270492137-00</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>fc8c6afb07ec5979e723bd03f9605b73</t>
+          <t>17b41f047b583d6c2cd61e5eb4ab8121</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>0bcb11a7-8901-4ada-a490-1db897384b02</t>
+          <t>25ef16ec-6641-462b-a607-de67040adc8c</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -1647,34 +1803,42 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6170656853", "EffectiveDate": "2026-08-21", "PolicyPaymentInfoList": [{"Amount": "893", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-08-21T10:34:21", "TransactionId": "c427a91f67ca2fa767df02b2bda78cc0:520346e774c87f1ddd061f9470830179", "TransactionNo": "TSIVrrpGnruz8L"}]}</t>
+          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6270518696", "EffectiveDate": "2026-09-18", "PolicyPaymentInfoList": [{"Amount": "6780", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-09-06T09:43:29", "TransactionId": "48c797525c6b36c8cd83957019380243:0629fffcbccd60b345338270454e4cad", "TransactionNo": "TYcCCQVWPaO15D"}]}</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>{"ihub.body": {"consumerAppTransId": "TSIVrrpGnruz8L", "gateway_txn_id": "TSIVrrpGnruz8L", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "893", "payment_id": "c427a91f67ca2fa767df02b2bda78cc0:520346e774c87f1ddd061f9470830179", "policy_start_date": "2026-08-21", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-08-21 10:34:21"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
+          <t>{"ihub.body": {"consumerAppTransId": "TYcCCQVWPaO15D", "gateway_txn_id": "TYcCCQVWPaO15D", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "6780", "payment_id": "48c797525c6b36c8cd83957019380243:0629fffcbccd60b345338270454e4cad", "policy_start_date": "2026-09-18", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-09-06 09:43:29"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "c48ef4d4a2ae245895f66e7bf09935bb:dd06bb0072f6e187e98682d1b28d4d84", "encrypted_policy_no": "89f98841847fe62323e18355bd0b52ad:b9a5268c177633c271273fa188aedfc2", "master_policy": "", "net_premium": 893, "nstp_id": "N500001950940", "nstp_stage": "completed", "payment_id": "5d110e87ae87d530b0b9cd157256fde7:063bf48bca342c36a87edf79ff657ca1", "payment_stage": "completed", "policy_id": "P500204183574", "policy_no": "6170719551-00", "product_id": "M300000000002", "proposal_no": "PR/26/6170656853", "proposal_stage": "completed", "quote_no": "QT/26/6176484797", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Success", "status": 200}</t>
+          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "c01b2f2962f6d14cfc009d16efadd96e:4138ab34992cba3a3b336225a44f523b", "encrypted_policy_no": "f48058b66ed5ad1d9cb4450690c11bf2:3e7101c23e4e3ab85dfcfb1769726cdf", "master_policy": "", "net_premium": 6780, "nstp_id": "N500002062524", "nstp_stage": "completed", "payment_id": "64ac7aacaf0871d2d52bd62e918e162e:ac30fb2533aafeeced2dd6148ffa6d10", "payment_stage": "completed", "policy_id": "P500211799173", "policy_no": "6270492137-00", "product_id": "M300000000001", "proposal_no": "PR/26/6270518696", "proposal_stage": "completed", "quote_no": "QT/26/6288383978", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>{"ClientRequestId": "0bcb11a7-8901-4ada-a490-1db897384b02", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6170719551-00", "CarrierProposalNo": "PR/26/6170656853", "CarrierQuoteRequestId": "QT/26/6176484797", "InspectionId": "N500001950940", "PaymentId": "5d110e87ae87d530b0b9cd157256fde7:063bf48bca342c36a87edf79ff657ca1", "requestId": "P500204183574"}, "ResultCode": 1, "TransactionType": 2003}</t>
+          <t>{"ClientRequestId": "25ef16ec-6641-462b-a607-de67040adc8c", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6270492137-00", "CarrierProposalNo": "PR/26/6270518696", "CarrierQuoteRequestId": "QT/26/6288383978", "InspectionId": "N500002062524", "PaymentId": "64ac7aacaf0871d2d52bd62e918e162e:ac30fb2533aafeeced2dd6148ffa6d10", "requestId": "P500211799173"}, "ResultCode": 1, "TransactionType": 2003}</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06T09:43:29</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23T18:54:09</t>
+          <t>2026-09-10T13:52:50</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -1682,17 +1846,17 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>6170725329-00</t>
+          <t>6270496952-00</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>60a059df8fcebe0a020e55affbfd87a5</t>
+          <t>5233fe39b5f32090ae3e5cd968e2c54c</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>437c430b-2785-432b-bf7e-f96c458512a9</t>
+          <t>66179c8c-1109-4ce9-8e6f-79e0b30c80ac</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -1707,34 +1871,42 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6170666328", "EffectiveDate": "2026-08-24", "PolicyPaymentInfoList": [{"Amount": "842", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-08-23T18:54:08", "TransactionId": "d4600d2da057a3e40340994d216ec15d:c5cd422c5142d6df20625b4bb9ff328d", "TransactionNo": "TTE64rmCQep66E"}]}</t>
+          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6270527707", "EffectiveDate": "2026-09-18", "PolicyPaymentInfoList": [{"Amount": "4905", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-09-10T13:52:49", "TransactionId": "f88f03bbf5b216e4c95b30175dc59c5d:291ad923d331d666a3c9195def086e3d", "TransactionNo": "TaGa9pMwTP9uBR"}]}</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>{"ihub.body": {"consumerAppTransId": "TTE64rmCQep66E", "gateway_txn_id": "TTE64rmCQep66E", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "842", "payment_id": "d4600d2da057a3e40340994d216ec15d:c5cd422c5142d6df20625b4bb9ff328d", "policy_start_date": "2026-08-24", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-08-23 18:54:08"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
+          <t>{"ihub.body": {"consumerAppTransId": "TaGa9pMwTP9uBR", "gateway_txn_id": "TaGa9pMwTP9uBR", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "4905", "payment_id": "f88f03bbf5b216e4c95b30175dc59c5d:291ad923d331d666a3c9195def086e3d", "policy_start_date": "2026-09-18", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-09-10 13:52:49"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "46c2f22cf5e9bbf328dc1cad0f064168:0bc7700ef571439cbf8645756c43f50f", "encrypted_policy_no": "772ef6e6b773d384ed8ba91c7139adf2:f7e1947dfc0303ed6a9211f3534e4b70", "master_policy": "", "net_premium": 842, "nstp_id": "N500001966970", "nstp_stage": "completed", "payment_id": "cda8b648ef0005b78a67ca5eff45f369:be4b478a2a977f9dab08281d4ff52ec9", "payment_stage": "completed", "policy_id": "P500205258244", "policy_no": "6170725329-00", "product_id": "M300000000002", "proposal_no": "PR/26/6170666328", "proposal_stage": "completed", "quote_no": "QT/26/6176550842", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
+          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "d51a67e088c5948f22fcf12b3cd64cec:c2abc50d2ecec167ee44bd2b7a8d1c33", "encrypted_policy_no": "3c9f770e0797182cbcb3ba57d268107d:0526243b1d54b9e1952e6a3059a4b399", "master_policy": "", "net_premium": 4905, "nstp_id": "N500002095899", "nstp_stage": "completed", "payment_id": "304e9193b00145afc4dd9b06fe9e9b66:83318fd96a4def7ce11360847ec986a0", "payment_stage": "completed", "policy_id": "P500213903422", "policy_no": "6270496952-00", "product_id": "M300000000001", "proposal_no": "PR/26/6270527707", "proposal_stage": "completed", "quote_no": "QT/26/6288692207", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>{"ClientRequestId": "437c430b-2785-432b-bf7e-f96c458512a9", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6170725329-00", "CarrierProposalNo": "PR/26/6170666328", "CarrierQuoteRequestId": "QT/26/6176550842", "InspectionId": "N500001966970", "PaymentId": "cda8b648ef0005b78a67ca5eff45f369:be4b478a2a977f9dab08281d4ff52ec9", "requestId": "P500205258244"}, "ResultCode": 1, "TransactionType": 2003}</t>
+          <t>{"ClientRequestId": "66179c8c-1109-4ce9-8e6f-79e0b30c80ac", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6270496952-00", "CarrierProposalNo": "PR/26/6270527707", "CarrierQuoteRequestId": "QT/26/6288692207", "InspectionId": "N500002095899", "PaymentId": "304e9193b00145afc4dd9b06fe9e9b66:83318fd96a4def7ce11360847ec986a0", "requestId": "P500213903422"}, "ResultCode": 1, "TransactionType": 2003}</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10T13:52:50</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26T10:35:44</t>
+          <t>2026-09-11T22:21:39</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -1742,17 +1914,17 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>6270479230-00</t>
+          <t>6170774054-00</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>515b7101c3e0e0a55571c0a407b51533</t>
+          <t>cab0f3696043b551d5b07847d2965a49</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>6b083cdc-67bd-4a1f-8905-96a696ca3c6b</t>
+          <t>34aa4c28-7d1c-4f1c-a53e-afd1bc1f21e7</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -1767,34 +1939,42 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6270495617", "EffectiveDate": "2026-09-02", "PolicyPaymentInfoList": [{"Amount": "8367", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-08-26T10:35:43", "TransactionId": "242b54330fd1c4db260cc8ec72936dde:8dbf8f8c09f4d4a7d21a659aecc326f3", "TransactionNo": "TUHCwfpI0VAVxC"}]}</t>
+          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6170760499", "EffectiveDate": "2026-09-12", "PolicyPaymentInfoList": [{"Amount": "843", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-09-11T22:21:39", "TransactionId": "e6c412fac45e6fc3b29e138265f4b2cc:8eaca3a73248c19714e3d09cb0ee4f5f", "TransactionNo": "Tanme4X5OCVJWw"}]}</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>{"ihub.body": {"consumerAppTransId": "TUHCwfpI0VAVxC", "gateway_txn_id": "TUHCwfpI0VAVxC", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "8367", "payment_id": "242b54330fd1c4db260cc8ec72936dde:8dbf8f8c09f4d4a7d21a659aecc326f3", "policy_start_date": "2026-09-02", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-08-26 10:35:43"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
+          <t>{"ihub.body": {"consumerAppTransId": "Tanme4X5OCVJWw", "gateway_txn_id": "Tanme4X5OCVJWw", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "843", "payment_id": "e6c412fac45e6fc3b29e138265f4b2cc:8eaca3a73248c19714e3d09cb0ee4f5f", "policy_start_date": "2026-09-12", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-09-11 22:21:39"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "d1d56bfda9ff92498d28047dfaadbba3:c5857debffbb2d2951df9bd221a100d5", "encrypted_policy_no": "5582bf7528d6f4a7e29a7f5f84b1c2a5:ed73e1c599ba3999879f10e120586999", "master_policy": "", "net_premium": 8367, "nstp_id": "N500001983446", "nstp_stage": "completed", "payment_id": "30beee7616b8dafb65cbf1c79e6a2aa5:c1328db2403f3db3eeaf22021825a571", "payment_stage": "completed", "policy_id": "P500206383696", "policy_no": "6270479230-00", "product_id": "M300000000001", "proposal_no": "PR/26/6270495617", "proposal_stage": "completed", "quote_no": "QT/26/6287576616", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
+          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "3a7a1448bb13e54c439a36f8e59650c8:e81c466e9362422add70f48dea4b009a", "encrypted_policy_no": "3000b350a2c0483d48a273503a465c1f:a6cd2f8768a38615c90b0dc4b1fe8ce7", "master_policy": "", "net_premium": 843, "nstp_id": "N500002107846", "nstp_stage": "completed", "payment_id": "f0912011e0bbbe477dd74a1da4e54a8a:6d85517e8659746c5f7f02419ccb16fd", "payment_stage": "completed", "policy_id": "P500214604006", "policy_no": "6170774054-00", "product_id": "M300000000002", "proposal_no": "PR/26/6170760499", "proposal_stage": "completed", "quote_no": "QT/26/6177113368", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>{"ClientRequestId": "6b083cdc-67bd-4a1f-8905-96a696ca3c6b", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6270479230-00", "CarrierProposalNo": "PR/26/6270495617", "CarrierQuoteRequestId": "QT/26/6287576616", "InspectionId": "N500001983446", "PaymentId": "30beee7616b8dafb65cbf1c79e6a2aa5:c1328db2403f3db3eeaf22021825a571", "requestId": "P500206383696"}, "ResultCode": 1, "TransactionType": 2003}</t>
+          <t>{"ClientRequestId": "34aa4c28-7d1c-4f1c-a53e-afd1bc1f21e7", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6170774054-00", "CarrierProposalNo": "PR/26/6170760499", "CarrierQuoteRequestId": "QT/26/6177113368", "InspectionId": "N500002107846", "PaymentId": "f0912011e0bbbe477dd74a1da4e54a8a:6d85517e8659746c5f7f02419ccb16fd", "requestId": "P500214604006"}, "ResultCode": 1, "TransactionType": 2003}</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11T22:21:41</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26T10:35:45</t>
+          <t>2026-09-18T15:50:27</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -1802,17 +1982,17 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>6270479230-00</t>
+          <t>6270505515-00</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>f3533000fd3dd5b5f5c85b6bf984504b</t>
+          <t>f954badefbe8e5c3b22c84a310061825</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>a5b74aa4-28cd-44a0-b2f3-95c8d03f0c5d</t>
+          <t>b4d4a9cf-ebb4-46ed-95d7-9ab62f423c12</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -1827,34 +2007,42 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6270495617", "EffectiveDate": "2026-09-02", "PolicyPaymentInfoList": [{"Amount": "8367", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-08-26T10:35:44", "TransactionId": "242b54330fd1c4db260cc8ec72936dde:8dbf8f8c09f4d4a7d21a659aecc326f3", "TransactionNo": "TUHCwfpI0VAVxC"}]}</t>
+          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6270543572", "EffectiveDate": "2026-09-20", "PolicyPaymentInfoList": [{"Amount": "13686", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-09-18T15:50:26", "TransactionId": "1d51850101b7b62157b0aa29ba399b89:36bdcb9ce4aa3f2b514ef688aea28d2e", "TransactionNo": "TdSrGXnXjr0YkF"}]}</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>{"ihub.body": {"consumerAppTransId": "TUHCwfpI0VAVxC", "gateway_txn_id": "TUHCwfpI0VAVxC", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "8367", "payment_id": "242b54330fd1c4db260cc8ec72936dde:8dbf8f8c09f4d4a7d21a659aecc326f3", "policy_start_date": "2026-09-02", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-08-26 10:35:44"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
+          <t>{"ihub.body": {"consumerAppTransId": "TdSrGXnXjr0YkF", "gateway_txn_id": "TdSrGXnXjr0YkF", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "13686", "payment_id": "1d51850101b7b62157b0aa29ba399b89:36bdcb9ce4aa3f2b514ef688aea28d2e", "policy_start_date": "2026-09-20", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-09-18 15:50:26"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "685f85ea93f68cf2aa7c01e5c94df2c0:7bec15158d2120396bfe28dc0cb1830b", "encrypted_policy_no": "f9870179b91f5fd91fef5068280d0493:6a944d349111370eec47d772cc5bbd45", "master_policy": "", "net_premium": 8367, "nstp_id": "N500001983446", "nstp_stage": "completed", "payment_id": "f54a76991274b74ed1c7d19f02f5ad7c:6a48c88cc7b66acc1a0f0fef18d56499", "payment_stage": "completed", "policy_id": "P500206383696", "policy_no": "6270479230-00", "product_id": "M300000000001", "proposal_no": "PR/26/6270495617", "proposal_stage": "completed", "quote_no": "QT/26/6287576616", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Success", "status": 200}</t>
+          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "75618e62c3d3e3c9aa1944335c1b7cc2:cddf755fd3658f2e4c79064242fee0cc", "encrypted_policy_no": "84318b721a57ff927b7851af6f5e0e70:3514711d9d81c6a57bfcd43e7cd7fb02", "master_policy": "", "net_premium": 13686, "nstp_id": "N500002152871", "nstp_stage": "completed", "payment_id": "b4b1f93003e219299e4eb8c933f9bb77:3dad9341a47b3e6f0ed94c47fbaaec08", "payment_stage": "completed", "policy_id": "P500217712112", "policy_no": "6270505515-00", "product_id": "M300000000001", "proposal_no": "PR/26/6270543572", "proposal_stage": "completed", "quote_no": "QT/26/6289281455", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>{"ClientRequestId": "a5b74aa4-28cd-44a0-b2f3-95c8d03f0c5d", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6270479230-00", "CarrierProposalNo": "PR/26/6270495617", "CarrierQuoteRequestId": "QT/26/6287576616", "InspectionId": "N500001983446", "PaymentId": "f54a76991274b74ed1c7d19f02f5ad7c:6a48c88cc7b66acc1a0f0fef18d56499", "requestId": "P500206383696"}, "ResultCode": 1, "TransactionType": 2003}</t>
+          <t>{"ClientRequestId": "b4d4a9cf-ebb4-46ed-95d7-9ab62f423c12", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6270505515-00", "CarrierProposalNo": "PR/26/6270543572", "CarrierQuoteRequestId": "QT/26/6289281455", "InspectionId": "N500002152871", "PaymentId": "b4b1f93003e219299e4eb8c933f9bb77:3dad9341a47b3e6f0ed94c47fbaaec08", "requestId": "P500217712112"}, "ResultCode": 1, "TransactionType": 2003}</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T15:50:27</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31T20:37:04</t>
+          <t>2026-10-02T13:05:57</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -1862,17 +2050,17 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>6170743506-00</t>
+          <t>6170827506-00</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>d9fbbfaeefd5d4334975b3b277229adb</t>
+          <t>688ec5985b4f03b9afb18df13daf72e3</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>f23871d4-ec7c-4c9c-a87c-70461144ac55</t>
+          <t>d1185f70-2198-4dc0-9ef0-97eabc8c806a</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -1887,682 +2075,30 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6170701071", "EffectiveDate": "2026-09-01", "PolicyPaymentInfoList": [{"Amount": "1285", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-08-31T20:37:03", "TransactionId": "d4abc8259e09ee9f4b2591a083cf720c:adf5184d95b9d62eb21cff3bac25182e", "TransactionNo": "TWQ7vcNMkcMtIL"}]}</t>
+          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6170861515", "EffectiveDate": "2026-10-03", "PolicyPaymentInfoList": [{"Amount": "1612", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-10-02T13:05:57", "TransactionId": "ab3e54fcc31c0864b6ec51a9ba01cb49:db73e31e352a90d07558a116ed8d8dbe", "TransactionNo": "TixXDhDKMVYhzF"}]}</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>{"ihub.body": {"consumerAppTransId": "TWQ7vcNMkcMtIL", "gateway_txn_id": "TWQ7vcNMkcMtIL", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "1285", "payment_id": "d4abc8259e09ee9f4b2591a083cf720c:adf5184d95b9d62eb21cff3bac25182e", "policy_start_date": "2026-09-01", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-08-31 20:37:03"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
+          <t>{"ihub.body": {"consumerAppTransId": "TixXDhDKMVYhzF", "gateway_txn_id": "TixXDhDKMVYhzF", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "1612", "payment_id": "ab3e54fcc31c0864b6ec51a9ba01cb49:db73e31e352a90d07558a116ed8d8dbe", "policy_start_date": "2026-10-03", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-10-02 13:05:57"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "ddd99c20a764e8ac0a07bca010c22021:14c214413eb50bbb7e9d831ee5e6df5a", "encrypted_policy_no": "c592381ad71e0b4d1956f30dff984aee:b1fc13ef179c008f1bb016d30c0a28ad", "master_policy": "", "net_premium": 1285, "nstp_id": "N500002021467", "nstp_stage": "completed", "payment_id": "afb898ed25b77e8c5edf008a91f5cb4f:6ae4e65047f0c160d3d98501e70f3058", "payment_stage": "completed", "policy_id": "P500209010887", "policy_no": "6170743506-00", "product_id": "M300000000002", "proposal_no": "PR/26/6170701071", "proposal_stage": "completed", "quote_no": "QT/26/6176761122", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
+          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "e1d45dddb599c2b47cf6cbdc2d972d46:5a73985bc0a7ba3d2f681de7bfcfff8d", "encrypted_policy_no": "66beee28f4aa733ebb17335aa918a4c0:00be83c5259ada617efc11e52498c8db", "master_policy": "", "net_premium": 1612, "nstp_id": "N500002256373", "nstp_stage": "completed", "payment_id": "d9a45fdbd87b3d816cfb64f8f4f42eb6:6200fe791d1eb0eef642375abaa8f631", "payment_stage": "completed", "policy_id": "P500224964822", "policy_no": "6170827506-00", "product_id": "M300000000002", "proposal_no": "PR/26/6170861515", "proposal_stage": "completed", "quote_no": "QT/26/6177758127", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>{"ClientRequestId": "f23871d4-ec7c-4c9c-a87c-70461144ac55", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6170743506-00", "CarrierProposalNo": "PR/26/6170701071", "CarrierQuoteRequestId": "QT/26/6176761122", "InspectionId": "N500002021467", "PaymentId": "afb898ed25b77e8c5edf008a91f5cb4f:6ae4e65047f0c160d3d98501e70f3058", "requestId": "P500209010887"}, "ResultCode": 1, "TransactionType": 2003}</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-31T20:37:06</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="n">
-        <v>2003</v>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>6170743506-00</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>49b3e8099d6ed0758f52b0faab497751</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>828ee394-5953-45bb-a45e-d6e70e9c5cfe</t>
-        </is>
-      </c>
-      <c r="G25" s="2" t="inlineStr">
-        <is>
-          <t>tataaig.motor.issuepolicy.url</t>
-        </is>
-      </c>
-      <c r="H25" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I25" s="2" t="inlineStr">
-        <is>
-          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6170701071", "EffectiveDate": "2026-09-01", "PolicyPaymentInfoList": [{"Amount": "1285", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-08-31T20:37:05", "TransactionId": "d4abc8259e09ee9f4b2591a083cf720c:adf5184d95b9d62eb21cff3bac25182e", "TransactionNo": "TWQ7vcNMkcMtIL"}]}</t>
-        </is>
-      </c>
-      <c r="J25" s="2" t="inlineStr">
-        <is>
-          <t>{"ihub.body": {"consumerAppTransId": "TWQ7vcNMkcMtIL", "gateway_txn_id": "TWQ7vcNMkcMtIL", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "1285", "payment_id": "d4abc8259e09ee9f4b2591a083cf720c:adf5184d95b9d62eb21cff3bac25182e", "policy_start_date": "2026-09-01", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-08-31 20:37:05"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
-        </is>
-      </c>
-      <c r="K25" s="2" t="inlineStr">
-        <is>
-          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "6a223ab9715ac9ab4120e89ea6dff460:a58e32f7a3f283df46ec68eb8aba63ca", "encrypted_policy_no": "6678af8de227f73b119b9d85dfa7d3b4:890717077f1996aa23ee6d108c05b4f6", "master_policy": "", "net_premium": 1285, "nstp_id": "N500002021467", "nstp_stage": "completed", "payment_id": "609d733a8cc650fb89ad986bded86080:92d6d7ad2a03fd8f473a2e0ef81b4a8b", "payment_stage": "completed", "policy_id": "P500209010887", "policy_no": "6170743506-00", "product_id": "M300000000002", "proposal_no": "PR/26/6170701071", "proposal_stage": "completed", "quote_no": "QT/26/6176761122", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Success", "status": 200}</t>
-        </is>
-      </c>
-      <c r="L25" s="2" t="inlineStr">
-        <is>
-          <t>{"ClientRequestId": "828ee394-5953-45bb-a45e-d6e70e9c5cfe", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6170743506-00", "CarrierProposalNo": "PR/26/6170701071", "CarrierQuoteRequestId": "QT/26/6176761122", "InspectionId": "N500002021467", "PaymentId": "609d733a8cc650fb89ad986bded86080:92d6d7ad2a03fd8f473a2e0ef81b4a8b", "requestId": "P500209010887"}, "ResultCode": 1, "TransactionType": 2003}</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-02T04:13:05</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="n">
-        <v>2003</v>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>6170746652-00</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>5a9555ac25de494af5adadb738cdab49</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>355bf614-8c68-4f8a-804b-6f2ed1505db1</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="inlineStr">
-        <is>
-          <t>tataaig.motor.issuepolicy.url</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6170706695", "EffectiveDate": "2026-09-03", "PolicyPaymentInfoList": [{"Amount": "1374", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-09-02T04:13:04", "TransactionId": "45a72cc153b5f202b926b37119a4de45:026f6dd545f62a770eb1b2d58a3eb37d", "TransactionNo": "TWwQXfsLqZhlas"}]}</t>
-        </is>
-      </c>
-      <c r="J26" s="2" t="inlineStr">
-        <is>
-          <t>{"ihub.body": {"consumerAppTransId": "TWwQXfsLqZhlas", "gateway_txn_id": "TWwQXfsLqZhlas", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "1374", "payment_id": "45a72cc153b5f202b926b37119a4de45:026f6dd545f62a770eb1b2d58a3eb37d", "policy_start_date": "2026-09-03", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-09-02 04:13:04"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
-        </is>
-      </c>
-      <c r="K26" s="2" t="inlineStr">
-        <is>
-          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "02b9a27d0c4d5990caf6b64c58b7f121:40d017d5f41614a76329f00884b7a9fa", "encrypted_policy_no": "17e32c558a1c4a9c8eb7f6d1b7662a82:b3835c140178c5c192b59f5d145ee344", "master_policy": "", "net_premium": 1374, "nstp_id": "N500002029991", "nstp_stage": "completed", "payment_id": "dadf53813b5f1be63dd0c32803d3ec67:8ed8a861e045e35058a141e6ee691965", "payment_stage": "completed", "policy_id": "P500209687513", "policy_no": "6170746652-00", "product_id": "M300000000002", "proposal_no": "PR/26/6170706695", "proposal_stage": "completed", "quote_no": "QT/26/6176796168", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
-        </is>
-      </c>
-      <c r="L26" s="2" t="inlineStr">
-        <is>
-          <t>{"ClientRequestId": "355bf614-8c68-4f8a-804b-6f2ed1505db1", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6170746652-00", "CarrierProposalNo": "PR/26/6170706695", "CarrierQuoteRequestId": "QT/26/6176796168", "InspectionId": "N500002029991", "PaymentId": "dadf53813b5f1be63dd0c32803d3ec67:8ed8a861e045e35058a141e6ee691965", "requestId": "P500209687513"}, "ResultCode": 1, "TransactionType": 2003}</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-02T04:13:06</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="n">
-        <v>2003</v>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>6170746652-00</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>5c43c356de8d5a62efcec414d7015cfc</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>050144b4-fbc7-4bde-b85e-8996cc433395</t>
-        </is>
-      </c>
-      <c r="G27" s="2" t="inlineStr">
-        <is>
-          <t>tataaig.motor.issuepolicy.url</t>
-        </is>
-      </c>
-      <c r="H27" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I27" s="2" t="inlineStr">
-        <is>
-          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6170706695", "EffectiveDate": "2026-09-03", "PolicyPaymentInfoList": [{"Amount": "1374", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-09-02T04:13:05", "TransactionId": "45a72cc153b5f202b926b37119a4de45:026f6dd545f62a770eb1b2d58a3eb37d", "TransactionNo": "TWwQXfsLqZhlas"}]}</t>
-        </is>
-      </c>
-      <c r="J27" s="2" t="inlineStr">
-        <is>
-          <t>{"ihub.body": {"consumerAppTransId": "TWwQXfsLqZhlas", "gateway_txn_id": "TWwQXfsLqZhlas", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "1374", "payment_id": "45a72cc153b5f202b926b37119a4de45:026f6dd545f62a770eb1b2d58a3eb37d", "policy_start_date": "2026-09-03", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-09-02 04:13:05"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
-        </is>
-      </c>
-      <c r="K27" s="2" t="inlineStr">
-        <is>
-          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "d8c3bd60a43949addbacac47a11acdf5:768416317045b7421279c5f915a2eb4c", "encrypted_policy_no": "295d1c17c8bc7b4c691642352b59ff33:d0f105913e82575d55e471e07e3284fe", "master_policy": "", "net_premium": 1374, "nstp_id": "N500002029991", "nstp_stage": "completed", "payment_id": "2d726b6069684bd5e1a2d588cf019e5d:64a092d14b1e179a25253a80546fa32c", "payment_stage": "completed", "policy_id": "P500209687513", "policy_no": "6170746652-00", "product_id": "M300000000002", "proposal_no": "PR/26/6170706695", "proposal_stage": "completed", "quote_no": "QT/26/6176796168", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Success", "status": 200}</t>
-        </is>
-      </c>
-      <c r="L27" s="2" t="inlineStr">
-        <is>
-          <t>{"ClientRequestId": "050144b4-fbc7-4bde-b85e-8996cc433395", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6170746652-00", "CarrierProposalNo": "PR/26/6170706695", "CarrierQuoteRequestId": "QT/26/6176796168", "InspectionId": "N500002029991", "PaymentId": "2d726b6069684bd5e1a2d588cf019e5d:64a092d14b1e179a25253a80546fa32c", "requestId": "P500209687513"}, "ResultCode": 1, "TransactionType": 2003}</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-02T15:54:22</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="n">
-        <v>2003</v>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>6170748395-00</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>ea722230d5dea0c06b03978d1350556c</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>b07934b8-dca3-48a6-88b8-6cb870adb157</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>tataaig.motor.issuepolicy.url</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I28" s="2" t="inlineStr">
-        <is>
-          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6170710217", "EffectiveDate": "2026-09-03", "PolicyPaymentInfoList": [{"Amount": "843", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-09-02T15:54:21", "TransactionId": "63dc00f0a7a0b038fb239d8af346dc1a:bff2effcd009a9b2c1e0747857aa2bd6", "TransactionNo": "TX8NHVzZdTLOoz"}]}</t>
-        </is>
-      </c>
-      <c r="J28" s="2" t="inlineStr">
-        <is>
-          <t>{"ihub.body": {"consumerAppTransId": "TX8NHVzZdTLOoz", "gateway_txn_id": "TX8NHVzZdTLOoz", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "843", "payment_id": "63dc00f0a7a0b038fb239d8af346dc1a:bff2effcd009a9b2c1e0747857aa2bd6", "policy_start_date": "2026-09-03", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-09-02 15:54:21"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
-        </is>
-      </c>
-      <c r="K28" s="2" t="inlineStr">
-        <is>
-          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "f883b4121427000b1a474f874343e7c9:af0986d46ed85850b236bae29738d6f9", "encrypted_policy_no": "0ba2a8306f35c3ff6a24c5b1bde6c2ff:0463ee2ed44e76183b8f06509043c497", "master_policy": "", "net_premium": 843, "nstp_id": "N500002035031", "nstp_stage": "completed", "payment_id": "43b9cf968f756b3023d48605cc8aba49:e8a5c497444a2e0edc43f533a611356b", "payment_stage": "completed", "policy_id": "P500209987686", "policy_no": "6170748395-00", "product_id": "M300000000002", "proposal_no": "PR/26/6170710217", "proposal_stage": "completed", "quote_no": "QT/26/6176815685", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
-        </is>
-      </c>
-      <c r="L28" s="2" t="inlineStr">
-        <is>
-          <t>{"ClientRequestId": "b07934b8-dca3-48a6-88b8-6cb870adb157", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6170748395-00", "CarrierProposalNo": "PR/26/6170710217", "CarrierQuoteRequestId": "QT/26/6176815685", "InspectionId": "N500002035031", "PaymentId": "43b9cf968f756b3023d48605cc8aba49:e8a5c497444a2e0edc43f533a611356b", "requestId": "P500209987686"}, "ResultCode": 1, "TransactionType": 2003}</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-02T15:54:23</t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="n">
-        <v>2003</v>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>6170748395-00</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>2d9ea4e05427f684d7afac152e36977b</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>6d33bd55-5a91-4b3b-86a6-a802945e54d3</t>
-        </is>
-      </c>
-      <c r="G29" s="2" t="inlineStr">
-        <is>
-          <t>tataaig.motor.issuepolicy.url</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I29" s="2" t="inlineStr">
-        <is>
-          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6170710217", "EffectiveDate": "2026-09-03", "PolicyPaymentInfoList": [{"Amount": "843", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-09-02T15:54:22", "TransactionId": "63dc00f0a7a0b038fb239d8af346dc1a:bff2effcd009a9b2c1e0747857aa2bd6", "TransactionNo": "TX8NHVzZdTLOoz"}]}</t>
-        </is>
-      </c>
-      <c r="J29" s="2" t="inlineStr">
-        <is>
-          <t>{"ihub.body": {"consumerAppTransId": "TX8NHVzZdTLOoz", "gateway_txn_id": "TX8NHVzZdTLOoz", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "843", "payment_id": "63dc00f0a7a0b038fb239d8af346dc1a:bff2effcd009a9b2c1e0747857aa2bd6", "policy_start_date": "2026-09-03", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-09-02 15:54:22"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
-        </is>
-      </c>
-      <c r="K29" s="2" t="inlineStr">
-        <is>
-          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "95be626a07c61979d201896275e4241a:d6fd51f5a3101199430b599ebe60ce76", "encrypted_policy_no": "36c1f36e11493eabdff8384aa04cf8f8:c471cfc2569b938bc35651608a3220ad", "master_policy": "", "net_premium": 843, "nstp_id": "N500002035031", "nstp_stage": "completed", "payment_id": "50589588bcfe6885fd2b963c14dfee63:91c5c41cdc56f4128fa50d5624595704", "payment_stage": "completed", "policy_id": "P500209987686", "policy_no": "6170748395-00", "product_id": "M300000000002", "proposal_no": "PR/26/6170710217", "proposal_stage": "completed", "quote_no": "QT/26/6176815685", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Success", "status": 200}</t>
-        </is>
-      </c>
-      <c r="L29" s="2" t="inlineStr">
-        <is>
-          <t>{"ClientRequestId": "6d33bd55-5a91-4b3b-86a6-a802945e54d3", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6170748395-00", "CarrierProposalNo": "PR/26/6170710217", "CarrierQuoteRequestId": "QT/26/6176815685", "InspectionId": "N500002035031", "PaymentId": "50589588bcfe6885fd2b963c14dfee63:91c5c41cdc56f4128fa50d5624595704", "requestId": "P500209987686"}, "ResultCode": 1, "TransactionType": 2003}</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-06</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-06T09:43:29</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="n">
-        <v>2003</v>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>6270492137-00</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>17b41f047b583d6c2cd61e5eb4ab8121</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>25ef16ec-6641-462b-a607-de67040adc8c</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t>tataaig.motor.issuepolicy.url</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I30" s="2" t="inlineStr">
-        <is>
-          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6270518696", "EffectiveDate": "2026-09-18", "PolicyPaymentInfoList": [{"Amount": "6780", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-09-06T09:43:29", "TransactionId": "48c797525c6b36c8cd83957019380243:0629fffcbccd60b345338270454e4cad", "TransactionNo": "TYcCCQVWPaO15D"}]}</t>
-        </is>
-      </c>
-      <c r="J30" s="2" t="inlineStr">
-        <is>
-          <t>{"ihub.body": {"consumerAppTransId": "TYcCCQVWPaO15D", "gateway_txn_id": "TYcCCQVWPaO15D", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "6780", "payment_id": "48c797525c6b36c8cd83957019380243:0629fffcbccd60b345338270454e4cad", "policy_start_date": "2026-09-18", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-09-06 09:43:29"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
-        </is>
-      </c>
-      <c r="K30" s="2" t="inlineStr">
-        <is>
-          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "c01b2f2962f6d14cfc009d16efadd96e:4138ab34992cba3a3b336225a44f523b", "encrypted_policy_no": "f48058b66ed5ad1d9cb4450690c11bf2:3e7101c23e4e3ab85dfcfb1769726cdf", "master_policy": "", "net_premium": 6780, "nstp_id": "N500002062524", "nstp_stage": "completed", "payment_id": "64ac7aacaf0871d2d52bd62e918e162e:ac30fb2533aafeeced2dd6148ffa6d10", "payment_stage": "completed", "policy_id": "P500211799173", "policy_no": "6270492137-00", "product_id": "M300000000001", "proposal_no": "PR/26/6270518696", "proposal_stage": "completed", "quote_no": "QT/26/6288383978", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
-        </is>
-      </c>
-      <c r="L30" s="2" t="inlineStr">
-        <is>
-          <t>{"ClientRequestId": "25ef16ec-6641-462b-a607-de67040adc8c", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6270492137-00", "CarrierProposalNo": "PR/26/6270518696", "CarrierQuoteRequestId": "QT/26/6288383978", "InspectionId": "N500002062524", "PaymentId": "64ac7aacaf0871d2d52bd62e918e162e:ac30fb2533aafeeced2dd6148ffa6d10", "requestId": "P500211799173"}, "ResultCode": 1, "TransactionType": 2003}</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-10</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-10T13:52:50</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="n">
-        <v>2003</v>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>6270496952-00</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>5233fe39b5f32090ae3e5cd968e2c54c</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>66179c8c-1109-4ce9-8e6f-79e0b30c80ac</t>
-        </is>
-      </c>
-      <c r="G31" s="2" t="inlineStr">
-        <is>
-          <t>tataaig.motor.issuepolicy.url</t>
-        </is>
-      </c>
-      <c r="H31" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I31" s="2" t="inlineStr">
-        <is>
-          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6270527707", "EffectiveDate": "2026-09-18", "PolicyPaymentInfoList": [{"Amount": "4905", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-09-10T13:52:49", "TransactionId": "f88f03bbf5b216e4c95b30175dc59c5d:291ad923d331d666a3c9195def086e3d", "TransactionNo": "TaGa9pMwTP9uBR"}]}</t>
-        </is>
-      </c>
-      <c r="J31" s="2" t="inlineStr">
-        <is>
-          <t>{"ihub.body": {"consumerAppTransId": "TaGa9pMwTP9uBR", "gateway_txn_id": "TaGa9pMwTP9uBR", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "4905", "payment_id": "f88f03bbf5b216e4c95b30175dc59c5d:291ad923d331d666a3c9195def086e3d", "policy_start_date": "2026-09-18", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-09-10 13:52:49"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
-        </is>
-      </c>
-      <c r="K31" s="2" t="inlineStr">
-        <is>
-          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "d51a67e088c5948f22fcf12b3cd64cec:c2abc50d2ecec167ee44bd2b7a8d1c33", "encrypted_policy_no": "3c9f770e0797182cbcb3ba57d268107d:0526243b1d54b9e1952e6a3059a4b399", "master_policy": "", "net_premium": 4905, "nstp_id": "N500002095899", "nstp_stage": "completed", "payment_id": "304e9193b00145afc4dd9b06fe9e9b66:83318fd96a4def7ce11360847ec986a0", "payment_stage": "completed", "policy_id": "P500213903422", "policy_no": "6270496952-00", "product_id": "M300000000001", "proposal_no": "PR/26/6270527707", "proposal_stage": "completed", "quote_no": "QT/26/6288692207", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
-        </is>
-      </c>
-      <c r="L31" s="2" t="inlineStr">
-        <is>
-          <t>{"ClientRequestId": "66179c8c-1109-4ce9-8e6f-79e0b30c80ac", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6270496952-00", "CarrierProposalNo": "PR/26/6270527707", "CarrierQuoteRequestId": "QT/26/6288692207", "InspectionId": "N500002095899", "PaymentId": "304e9193b00145afc4dd9b06fe9e9b66:83318fd96a4def7ce11360847ec986a0", "requestId": "P500213903422"}, "ResultCode": 1, "TransactionType": 2003}</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11T22:21:39</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="n">
-        <v>2003</v>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>6170774054-00</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>cab0f3696043b551d5b07847d2965a49</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>34aa4c28-7d1c-4f1c-a53e-afd1bc1f21e7</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="inlineStr">
-        <is>
-          <t>tataaig.motor.issuepolicy.url</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I32" s="2" t="inlineStr">
-        <is>
-          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6170760499", "EffectiveDate": "2026-09-12", "PolicyPaymentInfoList": [{"Amount": "843", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-09-11T22:21:39", "TransactionId": "e6c412fac45e6fc3b29e138265f4b2cc:8eaca3a73248c19714e3d09cb0ee4f5f", "TransactionNo": "Tanme4X5OCVJWw"}]}</t>
-        </is>
-      </c>
-      <c r="J32" s="2" t="inlineStr">
-        <is>
-          <t>{"ihub.body": {"consumerAppTransId": "Tanme4X5OCVJWw", "gateway_txn_id": "Tanme4X5OCVJWw", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "843", "payment_id": "e6c412fac45e6fc3b29e138265f4b2cc:8eaca3a73248c19714e3d09cb0ee4f5f", "policy_start_date": "2026-09-12", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-09-11 22:21:39"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
-        </is>
-      </c>
-      <c r="K32" s="2" t="inlineStr">
-        <is>
-          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "3a7a1448bb13e54c439a36f8e59650c8:e81c466e9362422add70f48dea4b009a", "encrypted_policy_no": "3000b350a2c0483d48a273503a465c1f:a6cd2f8768a38615c90b0dc4b1fe8ce7", "master_policy": "", "net_premium": 843, "nstp_id": "N500002107846", "nstp_stage": "completed", "payment_id": "f0912011e0bbbe477dd74a1da4e54a8a:6d85517e8659746c5f7f02419ccb16fd", "payment_stage": "completed", "policy_id": "P500214604006", "policy_no": "6170774054-00", "product_id": "M300000000002", "proposal_no": "PR/26/6170760499", "proposal_stage": "completed", "quote_no": "QT/26/6177113368", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
-        </is>
-      </c>
-      <c r="L32" s="2" t="inlineStr">
-        <is>
-          <t>{"ClientRequestId": "34aa4c28-7d1c-4f1c-a53e-afd1bc1f21e7", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6170774054-00", "CarrierProposalNo": "PR/26/6170760499", "CarrierQuoteRequestId": "QT/26/6177113368", "InspectionId": "N500002107846", "PaymentId": "f0912011e0bbbe477dd74a1da4e54a8a:6d85517e8659746c5f7f02419ccb16fd", "requestId": "P500214604006"}, "ResultCode": 1, "TransactionType": 2003}</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11T22:21:41</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="n">
-        <v>2003</v>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>6170774054-00</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>c4adcd89d62685271157b41e6e9a8502</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>b2f3bba6-c40f-4c5b-9106-f377744aad2c</t>
-        </is>
-      </c>
-      <c r="G33" s="2" t="inlineStr">
-        <is>
-          <t>tataaig.motor.issuepolicy.url</t>
-        </is>
-      </c>
-      <c r="H33" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I33" s="2" t="inlineStr">
-        <is>
-          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6170760499", "EffectiveDate": "2026-09-12", "PolicyPaymentInfoList": [{"Amount": "843", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-09-11T22:21:40", "TransactionId": "e6c412fac45e6fc3b29e138265f4b2cc:8eaca3a73248c19714e3d09cb0ee4f5f", "TransactionNo": "Tanme4X5OCVJWw"}]}</t>
-        </is>
-      </c>
-      <c r="J33" s="2" t="inlineStr">
-        <is>
-          <t>{"ihub.body": {"consumerAppTransId": "Tanme4X5OCVJWw", "gateway_txn_id": "Tanme4X5OCVJWw", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "843", "payment_id": "e6c412fac45e6fc3b29e138265f4b2cc:8eaca3a73248c19714e3d09cb0ee4f5f", "policy_start_date": "2026-09-12", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-09-11 22:21:40"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
-        </is>
-      </c>
-      <c r="K33" s="2" t="inlineStr">
-        <is>
-          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "d9fa2f833d8279a20e580cc2a12add48:032f40dd3be9abb6b269da7a85f357e7", "encrypted_policy_no": "4a5f354a827913d8dea068b367382080:1073d97690680120e2830a822fe82813", "master_policy": "", "net_premium": 843, "nstp_id": "N500002107846", "nstp_stage": "completed", "payment_id": "92145953b67f101170cc6f2f67af9ffa:1ac6113c0f862fd13bdf385e83fbf5a8", "payment_stage": "completed", "policy_id": "P500214604006", "policy_no": "6170774054-00", "product_id": "M300000000002", "proposal_no": "PR/26/6170760499", "proposal_stage": "completed", "quote_no": "QT/26/6177113368", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Success", "status": 200}</t>
-        </is>
-      </c>
-      <c r="L33" s="2" t="inlineStr">
-        <is>
-          <t>{"ClientRequestId": "b2f3bba6-c40f-4c5b-9106-f377744aad2c", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6170774054-00", "CarrierProposalNo": "PR/26/6170760499", "CarrierQuoteRequestId": "QT/26/6177113368", "InspectionId": "N500002107846", "PaymentId": "92145953b67f101170cc6f2f67af9ffa:1ac6113c0f862fd13bdf385e83fbf5a8", "requestId": "P500214604006"}, "ResultCode": 1, "TransactionType": 2003}</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-18T15:50:27</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="n">
-        <v>2003</v>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>6270505515-00</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>f954badefbe8e5c3b22c84a310061825</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>b4d4a9cf-ebb4-46ed-95d7-9ab62f423c12</t>
-        </is>
-      </c>
-      <c r="G34" s="2" t="inlineStr">
-        <is>
-          <t>tataaig.motor.issuepolicy.url</t>
-        </is>
-      </c>
-      <c r="H34" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I34" s="2" t="inlineStr">
-        <is>
-          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6270543572", "EffectiveDate": "2026-09-20", "PolicyPaymentInfoList": [{"Amount": "13686", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-09-18T15:50:26", "TransactionId": "1d51850101b7b62157b0aa29ba399b89:36bdcb9ce4aa3f2b514ef688aea28d2e", "TransactionNo": "TdSrGXnXjr0YkF"}]}</t>
-        </is>
-      </c>
-      <c r="J34" s="2" t="inlineStr">
-        <is>
-          <t>{"ihub.body": {"consumerAppTransId": "TdSrGXnXjr0YkF", "gateway_txn_id": "TdSrGXnXjr0YkF", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "13686", "payment_id": "1d51850101b7b62157b0aa29ba399b89:36bdcb9ce4aa3f2b514ef688aea28d2e", "policy_start_date": "2026-09-20", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-09-18 15:50:26"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
-        </is>
-      </c>
-      <c r="K34" s="2" t="inlineStr">
-        <is>
-          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "75618e62c3d3e3c9aa1944335c1b7cc2:cddf755fd3658f2e4c79064242fee0cc", "encrypted_policy_no": "84318b721a57ff927b7851af6f5e0e70:3514711d9d81c6a57bfcd43e7cd7fb02", "master_policy": "", "net_premium": 13686, "nstp_id": "N500002152871", "nstp_stage": "completed", "payment_id": "b4b1f93003e219299e4eb8c933f9bb77:3dad9341a47b3e6f0ed94c47fbaaec08", "payment_stage": "completed", "policy_id": "P500217712112", "policy_no": "6270505515-00", "product_id": "M300000000001", "proposal_no": "PR/26/6270543572", "proposal_stage": "completed", "quote_no": "QT/26/6289281455", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
-        </is>
-      </c>
-      <c r="L34" s="2" t="inlineStr">
-        <is>
-          <t>{"ClientRequestId": "b4d4a9cf-ebb4-46ed-95d7-9ab62f423c12", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6270505515-00", "CarrierProposalNo": "PR/26/6270543572", "CarrierQuoteRequestId": "QT/26/6289281455", "InspectionId": "N500002152871", "PaymentId": "b4b1f93003e219299e4eb8c933f9bb77:3dad9341a47b3e6f0ed94c47fbaaec08", "requestId": "P500217712112"}, "ResultCode": 1, "TransactionType": 2003}</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
+          <t>{"ClientRequestId": "d1185f70-2198-4dc0-9ef0-97eabc8c806a", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6170827506-00", "CarrierProposalNo": "PR/26/6170861515", "CarrierQuoteRequestId": "QT/26/6177758127", "InspectionId": "N500002256373", "PaymentId": "d9a45fdbd87b3d816cfb64f8f4f42eb6:6200fe791d1eb0eef642375abaa8f631", "requestId": "P500224964822"}, "ResultCode": 1, "TransactionType": 2003}</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
         <is>
           <t>2026-10-02T13:05:57</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="n">
-        <v>2003</v>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>6170827506-00</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>688ec5985b4f03b9afb18df13daf72e3</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr">
-        <is>
-          <t>d1185f70-2198-4dc0-9ef0-97eabc8c806a</t>
-        </is>
-      </c>
-      <c r="G35" s="2" t="inlineStr">
-        <is>
-          <t>tataaig.motor.issuepolicy.url</t>
-        </is>
-      </c>
-      <c r="H35" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I35" s="2" t="inlineStr">
-        <is>
-          <t>{"CarrierCode": "25", "CarrierProposalNo": "PR/26/6170861515", "EffectiveDate": "2026-10-03", "PolicyPaymentInfoList": [{"Amount": "1612", "IsInstallment": "N", "PayModeCode": "ONLINE", "PaymentDate": "2026-10-02T13:05:57", "TransactionId": "ab3e54fcc31c0864b6ec51a9ba01cb49:db73e31e352a90d07558a116ed8d8dbe", "TransactionNo": "TixXDhDKMVYhzF"}]}</t>
-        </is>
-      </c>
-      <c r="J35" s="2" t="inlineStr">
-        <is>
-          <t>{"ihub.body": {"consumerAppTransId": "TixXDhDKMVYhzF", "gateway_txn_id": "TixXDhDKMVYhzF", "office_location_code": "lcode", "office_location_name": "lname", "payer_type": "Customer", "payment_amount": "1612", "payment_id": "ab3e54fcc31c0864b6ec51a9ba01cb49:db73e31e352a90d07558a116ed8d8dbe", "policy_start_date": "2026-10-03", "producer_code": "2958590000", "transactionStatus": "Success", "txn_start_time": "2026-10-02 13:05:57"}, "ihub.params": {"path": {"endpoints": "payment/online_response?product=Motor"}}}</t>
-        </is>
-      </c>
-      <c r="K35" s="2" t="inlineStr">
-        <is>
-          <t>{"data": [{"certificate_seq_no": "", "document_stage": "inprogress", "encrypted_policy_id": "e1d45dddb599c2b47cf6cbdc2d972d46:5a73985bc0a7ba3d2f681de7bfcfff8d", "encrypted_policy_no": "66beee28f4aa733ebb17335aa918a4c0:00be83c5259ada617efc11e52498c8db", "master_policy": "", "net_premium": 1612, "nstp_id": "N500002256373", "nstp_stage": "completed", "payment_id": "d9a45fdbd87b3d816cfb64f8f4f42eb6:6200fe791d1eb0eef642375abaa8f631", "payment_stage": "completed", "policy_id": "P500224964822", "policy_no": "6170827506-00", "product_id": "M300000000002", "proposal_no": "PR/26/6170861515", "proposal_stage": "completed", "quote_no": "QT/26/6177758127", "quote_stage": "completed", "verify_stage": "inprogress"}], "message_txt": "Payment completed", "status": 200}</t>
-        </is>
-      </c>
-      <c r="L35" s="2" t="inlineStr">
-        <is>
-          <t>{"ClientRequestId": "d1185f70-2198-4dc0-9ef0-97eabc8c806a", "CountryCode": "IND", "ProviderCode": "TATAAIG", "Result": {"CarrierCode": "25", "CarrierPolicyNo": "6170827506-00", "CarrierProposalNo": "PR/26/6170861515", "CarrierQuoteRequestId": "QT/26/6177758127", "InspectionId": "N500002256373", "PaymentId": "d9a45fdbd87b3d816cfb64f8f4f42eb6:6200fe791d1eb0eef642375abaa8f631", "requestId": "P500224964822"}, "ResultCode": 1, "TransactionType": 2003}</t>
         </is>
       </c>
     </row>

</xml_diff>